<commit_message>
Release v2.0.0: new search query, extend the index to 2026-09
- Full-text search for the rare-earth and shortage terms; articles of 100 to 1,999 words
- New source importance weights in config/sources.csv
- Index from 2008-01 to 2026-09; index.csv and index.xlsx hold the two standardized series
- README, CITATION.cff and CHANGELOG updated
</commit_message>
<xml_diff>
--- a/data/processed/index.xlsx
+++ b/data/processed/index.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F224"/>
+  <dimension ref="A1:D226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,20 +462,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>unstandardized</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>unstandardized weighted</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
           <t>standardized</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>standardized weighted</t>
         </is>
@@ -492,12 +482,6 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -512,12 +496,6 @@
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n"/>
@@ -530,12 +508,6 @@
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n"/>
@@ -548,12 +520,6 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n"/>
@@ -566,12 +532,6 @@
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n"/>
@@ -584,12 +544,6 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n"/>
@@ -602,12 +556,6 @@
       <c r="D8" t="n">
         <v>0</v>
       </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n"/>
@@ -620,12 +568,6 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n"/>
@@ -633,16 +575,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>9.178439125865477</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
+        <v>11.51392941433847</v>
       </c>
     </row>
     <row r="11">
@@ -656,12 +592,6 @@
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n"/>
@@ -674,12 +604,6 @@
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n"/>
@@ -692,12 +616,6 @@
       <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -707,16 +625,10 @@
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>28.98667030600534</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E14" t="n">
-        <v>54.06757666999513</v>
-      </c>
-      <c r="F14" t="n">
-        <v>9.987877969056045</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -730,12 +642,6 @@
       <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n"/>
@@ -748,12 +654,6 @@
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
@@ -766,12 +666,6 @@
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
@@ -784,12 +678,6 @@
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
@@ -802,12 +690,6 @@
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
@@ -820,12 +702,6 @@
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n"/>
@@ -838,12 +714,6 @@
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n"/>
@@ -851,16 +721,10 @@
         <v>9</v>
       </c>
       <c r="C22" t="n">
-        <v>4.104878959460642</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E22" t="n">
-        <v>6.842033308871132</v>
-      </c>
-      <c r="F22" t="n">
-        <v>8.925231348861518</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -869,16 +733,10 @@
         <v>10</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>3.454881659426192</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0</v>
+        <v>2.479273538095631</v>
       </c>
     </row>
     <row r="24">
@@ -892,12 +750,6 @@
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n"/>
@@ -910,12 +762,6 @@
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -925,16 +771,10 @@
         <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>9.487370809588889</v>
+        <v>41.81728610087828</v>
       </c>
       <c r="D26" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E26" t="n">
-        <v>124.5618198598366</v>
-      </c>
-      <c r="F26" t="n">
-        <v>128.9866471171744</v>
+        <v>44.35918369906828</v>
       </c>
     </row>
     <row r="27">
@@ -943,16 +783,10 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>12.24810491948888</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="n">
-        <v>0</v>
+        <v>9.169084245680017</v>
       </c>
     </row>
     <row r="28">
@@ -961,16 +795,10 @@
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>8.531097992394884</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="n">
-        <v>0</v>
+        <v>11.51392941433847</v>
       </c>
     </row>
     <row r="29">
@@ -979,16 +807,10 @@
         <v>4</v>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>11.89538647854219</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" t="n">
-        <v>0</v>
+        <v>22.45453984486278</v>
       </c>
     </row>
     <row r="30">
@@ -997,16 +819,10 @@
         <v>5</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>40.74350978635739</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" t="n">
-        <v>0</v>
+        <v>22.53454784319519</v>
       </c>
     </row>
     <row r="31">
@@ -1015,16 +831,10 @@
         <v>6</v>
       </c>
       <c r="C31" t="n">
-        <v>4.177070830756949</v>
+        <v>37.01325577200375</v>
       </c>
       <c r="D31" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E31" t="n">
-        <v>87.91025193247562</v>
-      </c>
-      <c r="F31" t="n">
-        <v>323.2752189457334</v>
+        <v>95.96794405468442</v>
       </c>
     </row>
     <row r="32">
@@ -1038,12 +848,6 @@
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="E32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n"/>
@@ -1051,16 +855,10 @@
         <v>8</v>
       </c>
       <c r="C33" t="n">
-        <v>14.0998839777979</v>
+        <v>41.56610491801685</v>
       </c>
       <c r="D33" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E33" t="n">
-        <v>84.71697368799741</v>
-      </c>
-      <c r="F33" t="n">
-        <v>63.73448125007216</v>
+        <v>32.54532128623082</v>
       </c>
     </row>
     <row r="34">
@@ -1069,16 +867,10 @@
         <v>9</v>
       </c>
       <c r="C34" t="n">
-        <v>14.67631333403033</v>
+        <v>122.8793525914728</v>
       </c>
       <c r="D34" t="n">
-        <v>127.6466013376886</v>
-      </c>
-      <c r="E34" t="n">
-        <v>113.4575856060316</v>
-      </c>
-      <c r="F34" t="n">
-        <v>156.5410646231054</v>
+        <v>186.0350167870397</v>
       </c>
     </row>
     <row r="35">
@@ -1087,16 +879,10 @@
         <v>10</v>
       </c>
       <c r="C35" t="n">
-        <v>74.45810661438166</v>
+        <v>79.78049106334339</v>
       </c>
       <c r="D35" t="n">
-        <v>287.2048530097993</v>
-      </c>
-      <c r="E35" t="n">
-        <v>242.0102454052046</v>
-      </c>
-      <c r="F35" t="n">
-        <v>251.2022263910697</v>
+        <v>94.67082555776153</v>
       </c>
     </row>
     <row r="36">
@@ -1105,16 +891,10 @@
         <v>11</v>
       </c>
       <c r="C36" t="n">
-        <v>69.78200446877463</v>
+        <v>120.797832310949</v>
       </c>
       <c r="D36" t="n">
-        <v>191.4699020065329</v>
-      </c>
-      <c r="E36" t="n">
-        <v>179.5640955192068</v>
-      </c>
-      <c r="F36" t="n">
-        <v>124.8375218297405</v>
+        <v>72.67441095647149</v>
       </c>
     </row>
     <row r="37">
@@ -1123,16 +903,10 @@
         <v>12</v>
       </c>
       <c r="C37" t="n">
-        <v>94.29525120683481</v>
+        <v>133.6139612685582</v>
       </c>
       <c r="D37" t="n">
-        <v>223.381552340955</v>
-      </c>
-      <c r="E37" t="n">
-        <v>515.2274672211088</v>
-      </c>
-      <c r="F37" t="n">
-        <v>579.116410040091</v>
+        <v>182.9147852679767</v>
       </c>
     </row>
     <row r="38">
@@ -1143,16 +917,10 @@
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>71.13338472774609</v>
+        <v>57.0143341332905</v>
       </c>
       <c r="D38" t="n">
-        <v>127.6466013376886</v>
-      </c>
-      <c r="E38" t="n">
-        <v>265.7832849757661</v>
-      </c>
-      <c r="F38" t="n">
-        <v>185.0940777068855</v>
+        <v>62.12628901580505</v>
       </c>
     </row>
     <row r="39">
@@ -1161,16 +929,10 @@
         <v>2</v>
       </c>
       <c r="C39" t="n">
-        <v>12.45978076444032</v>
+        <v>28.34374438379606</v>
       </c>
       <c r="D39" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E39" t="n">
-        <v>53.76100369856411</v>
-      </c>
-      <c r="F39" t="n">
-        <v>75.74805245004677</v>
+        <v>37.3696978698618</v>
       </c>
     </row>
     <row r="40">
@@ -1179,16 +941,10 @@
         <v>3</v>
       </c>
       <c r="C40" t="n">
-        <v>40.51209636226763</v>
+        <v>103.3354514560108</v>
       </c>
       <c r="D40" t="n">
-        <v>159.5582516721107</v>
-      </c>
-      <c r="E40" t="n">
-        <v>241.3861768336782</v>
-      </c>
-      <c r="F40" t="n">
-        <v>261.3799759158714</v>
+        <v>126.3911570090188</v>
       </c>
     </row>
     <row r="41">
@@ -1197,16 +953,10 @@
         <v>4</v>
       </c>
       <c r="C41" t="n">
-        <v>23.64257006289117</v>
+        <v>25.77887002476456</v>
       </c>
       <c r="D41" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E41" t="n">
-        <v>53.55109630386479</v>
-      </c>
-      <c r="F41" t="n">
-        <v>12.12853470204306</v>
+        <v>16.85412225235489</v>
       </c>
     </row>
     <row r="42">
@@ -1215,16 +965,10 @@
         <v>5</v>
       </c>
       <c r="C42" t="n">
-        <v>12.36976956281913</v>
+        <v>67.64628909121681</v>
       </c>
       <c r="D42" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E42" t="n">
-        <v>64.85353613002319</v>
-      </c>
-      <c r="F42" t="n">
-        <v>28.0741557762662</v>
+        <v>33.83527027586731</v>
       </c>
     </row>
     <row r="43">
@@ -1233,16 +977,10 @@
         <v>6</v>
       </c>
       <c r="C43" t="n">
-        <v>12.1703435099508</v>
+        <v>44.29437038248208</v>
       </c>
       <c r="D43" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E43" t="n">
-        <v>81.74794333027428</v>
-      </c>
-      <c r="F43" t="n">
-        <v>98.64347487078169</v>
+        <v>37.1914330116954</v>
       </c>
     </row>
     <row r="44">
@@ -1251,16 +989,10 @@
         <v>7</v>
       </c>
       <c r="C44" t="n">
-        <v>75.82903151417672</v>
+        <v>99.51422626170849</v>
       </c>
       <c r="D44" t="n">
-        <v>255.2932026753772</v>
-      </c>
-      <c r="E44" t="n">
-        <v>415.1054712212389</v>
-      </c>
-      <c r="F44" t="n">
-        <v>694.8008795254716</v>
+        <v>227.5726401264791</v>
       </c>
     </row>
     <row r="45">
@@ -1269,16 +1001,10 @@
         <v>8</v>
       </c>
       <c r="C45" t="n">
-        <v>80.17000132329345</v>
+        <v>40.46870780496606</v>
       </c>
       <c r="D45" t="n">
-        <v>127.6466013376886</v>
-      </c>
-      <c r="E45" t="n">
-        <v>315.3473615215103</v>
-      </c>
-      <c r="F45" t="n">
-        <v>103.1343118941334</v>
+        <v>16.17455788388394</v>
       </c>
     </row>
     <row r="46">
@@ -1287,16 +1013,10 @@
         <v>9</v>
       </c>
       <c r="C46" t="n">
-        <v>55.32184598030499</v>
+        <v>9.690567709919769</v>
       </c>
       <c r="D46" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E46" t="n">
-        <v>114.759348845996</v>
-      </c>
-      <c r="F46" t="n">
-        <v>37.34745618015791</v>
+        <v>6.826494886212494</v>
       </c>
     </row>
     <row r="47">
@@ -1305,16 +1025,10 @@
         <v>10</v>
       </c>
       <c r="C47" t="n">
-        <v>1.412259186164197</v>
+        <v>77.64168620845801</v>
       </c>
       <c r="D47" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E47" t="n">
-        <v>9.655720118903046</v>
-      </c>
-      <c r="F47" t="n">
-        <v>36.61043710727625</v>
+        <v>64.63323916011262</v>
       </c>
     </row>
     <row r="48">
@@ -1323,16 +1037,10 @@
         <v>11</v>
       </c>
       <c r="C48" t="n">
-        <v>18.85358681520687</v>
+        <v>143.6360183643897</v>
       </c>
       <c r="D48" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E48" t="n">
-        <v>133.1539419061284</v>
-      </c>
-      <c r="F48" t="n">
-        <v>74.52843016758334</v>
+        <v>115.2991092537007</v>
       </c>
     </row>
     <row r="49">
@@ -1341,16 +1049,10 @@
         <v>12</v>
       </c>
       <c r="C49" t="n">
-        <v>5.090875011029581</v>
+        <v>45.87797060792168</v>
       </c>
       <c r="D49" t="n">
-        <v>31.91165033442215</v>
-      </c>
-      <c r="E49" t="n">
-        <v>8.485496586077364</v>
-      </c>
-      <c r="F49" t="n">
-        <v>8.925231348861518</v>
+        <v>124.2529948527074</v>
       </c>
     </row>
     <row r="50">
@@ -1361,16 +1063,10 @@
         <v>1</v>
       </c>
       <c r="C50" t="n">
-        <v>21.18805711155279</v>
+        <v>174.8803014392545</v>
       </c>
       <c r="D50" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E50" t="n">
-        <v>390.2090677346644</v>
-      </c>
-      <c r="F50" t="n">
-        <v>157.6333850217771</v>
+        <v>78.16210863967638</v>
       </c>
     </row>
     <row r="51">
@@ -1379,16 +1075,10 @@
         <v>2</v>
       </c>
       <c r="C51" t="n">
-        <v>1.36057497608768</v>
+        <v>73.72014661828268</v>
       </c>
       <c r="D51" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E51" t="n">
-        <v>9.302351366230324</v>
-      </c>
-      <c r="F51" t="n">
-        <v>36.61043710727625</v>
+        <v>36.74336006110997</v>
       </c>
     </row>
     <row r="52">
@@ -1397,16 +1087,10 @@
         <v>3</v>
       </c>
       <c r="C52" t="n">
-        <v>56.74634091970923</v>
+        <v>195.715557245195</v>
       </c>
       <c r="D52" t="n">
-        <v>414.8514543474878</v>
-      </c>
-      <c r="E52" t="n">
-        <v>491.5961254153599</v>
-      </c>
-      <c r="F52" t="n">
-        <v>587.5183513162536</v>
+        <v>266.703200463893</v>
       </c>
     </row>
     <row r="53">
@@ -1415,16 +1099,10 @@
         <v>4</v>
       </c>
       <c r="C53" t="n">
-        <v>25.52280915350715</v>
+        <v>41.13177211930125</v>
       </c>
       <c r="D53" t="n">
-        <v>127.6466013376886</v>
-      </c>
-      <c r="E53" t="n">
-        <v>121.1526343854284</v>
-      </c>
-      <c r="F53" t="n">
-        <v>115.4408824094472</v>
+        <v>37.78796617910261</v>
       </c>
     </row>
     <row r="54">
@@ -1433,16 +1111,10 @@
         <v>5</v>
       </c>
       <c r="C54" t="n">
-        <v>3.834534925037421</v>
+        <v>44.03333451948032</v>
       </c>
       <c r="D54" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E54" t="n">
-        <v>113.5848355152307</v>
-      </c>
-      <c r="F54" t="n">
-        <v>158.6142892321014</v>
+        <v>63.82604189770095</v>
       </c>
     </row>
     <row r="55">
@@ -1451,16 +1123,10 @@
         <v>6</v>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>13.89925746049752</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
-      </c>
-      <c r="E55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" t="n">
-        <v>0</v>
+        <v>10.93895100748031</v>
       </c>
     </row>
     <row r="56">
@@ -1469,16 +1135,10 @@
         <v>7</v>
       </c>
       <c r="C56" t="n">
-        <v>0</v>
+        <v>46.92777665183239</v>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
-      </c>
-      <c r="E56" t="n">
-        <v>0</v>
-      </c>
-      <c r="F56" t="n">
-        <v>0</v>
+        <v>24.87939301185365</v>
       </c>
     </row>
     <row r="57">
@@ -1487,16 +1147,10 @@
         <v>8</v>
       </c>
       <c r="C57" t="n">
-        <v>27.23269752746837</v>
+        <v>57.83548184243602</v>
       </c>
       <c r="D57" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E57" t="n">
-        <v>202.7757876226624</v>
-      </c>
-      <c r="F57" t="n">
-        <v>80.028594348415</v>
+        <v>43.33396340050574</v>
       </c>
     </row>
     <row r="58">
@@ -1505,16 +1159,10 @@
         <v>9</v>
       </c>
       <c r="C58" t="n">
-        <v>1.088693919934326</v>
+        <v>4.2859619507581</v>
       </c>
       <c r="D58" t="n">
-        <v>31.91165033442215</v>
-      </c>
-      <c r="E58" t="n">
-        <v>7.443480551603997</v>
-      </c>
-      <c r="F58" t="n">
-        <v>36.61043710727625</v>
+        <v>21.8812208610486</v>
       </c>
     </row>
     <row r="59">
@@ -1523,16 +1171,10 @@
         <v>10</v>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>11.28369557861036</v>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
-      </c>
-      <c r="E59" t="n">
-        <v>0</v>
-      </c>
-      <c r="F59" t="n">
-        <v>0</v>
+        <v>46.24171526019283</v>
       </c>
     </row>
     <row r="60">
@@ -1541,16 +1183,10 @@
         <v>11</v>
       </c>
       <c r="C60" t="n">
-        <v>6.355609329955374</v>
+        <v>10.48465443076698</v>
       </c>
       <c r="D60" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E60" t="n">
-        <v>35.85977300389222</v>
-      </c>
-      <c r="F60" t="n">
-        <v>30.21238399390899</v>
+        <v>9.169084245680017</v>
       </c>
     </row>
     <row r="61">
@@ -1559,16 +1195,10 @@
         <v>12</v>
       </c>
       <c r="C61" t="n">
-        <v>5.63764121978234</v>
+        <v>0</v>
       </c>
       <c r="D61" t="n">
-        <v>31.91165033442215</v>
-      </c>
-      <c r="E61" t="n">
-        <v>9.396849307898696</v>
-      </c>
-      <c r="F61" t="n">
-        <v>8.925231348861518</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -1582,12 +1212,6 @@
         <v>0</v>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
-      </c>
-      <c r="E62" t="n">
-        <v>0</v>
-      </c>
-      <c r="F62" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1602,12 +1226,6 @@
       <c r="D63" t="n">
         <v>0</v>
       </c>
-      <c r="E63" t="n">
-        <v>0</v>
-      </c>
-      <c r="F63" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n"/>
@@ -1615,16 +1233,10 @@
         <v>3</v>
       </c>
       <c r="C64" t="n">
-        <v>4.898859415836008</v>
+        <v>237.6361409433172</v>
       </c>
       <c r="D64" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E64" t="n">
-        <v>351.5863735329119</v>
-      </c>
-      <c r="F64" t="n">
-        <v>384.301174587959</v>
+        <v>261.3877223923998</v>
       </c>
     </row>
     <row r="65">
@@ -1638,12 +1250,6 @@
       <c r="D65" t="n">
         <v>0</v>
       </c>
-      <c r="E65" t="n">
-        <v>0</v>
-      </c>
-      <c r="F65" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n"/>
@@ -1651,16 +1257,10 @@
         <v>5</v>
       </c>
       <c r="C66" t="n">
-        <v>11.70518922235571</v>
+        <v>34.91445766048764</v>
       </c>
       <c r="D66" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E66" t="n">
-        <v>61.36920403291622</v>
-      </c>
-      <c r="F66" t="n">
-        <v>28.0741557762662</v>
+        <v>16.57890708824532</v>
       </c>
     </row>
     <row r="67">
@@ -1674,12 +1274,6 @@
       <c r="D67" t="n">
         <v>0</v>
       </c>
-      <c r="E67" t="n">
-        <v>0</v>
-      </c>
-      <c r="F67" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n"/>
@@ -1692,12 +1286,6 @@
       <c r="D68" t="n">
         <v>0</v>
       </c>
-      <c r="E68" t="n">
-        <v>0</v>
-      </c>
-      <c r="F68" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n"/>
@@ -1710,12 +1298,6 @@
       <c r="D69" t="n">
         <v>0</v>
       </c>
-      <c r="E69" t="n">
-        <v>0</v>
-      </c>
-      <c r="F69" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n"/>
@@ -1728,12 +1310,6 @@
       <c r="D70" t="n">
         <v>0</v>
       </c>
-      <c r="E70" t="n">
-        <v>0</v>
-      </c>
-      <c r="F70" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n"/>
@@ -1741,16 +1317,10 @@
         <v>10</v>
       </c>
       <c r="C71" t="n">
-        <v>2.007399073056693</v>
+        <v>18.46262659676481</v>
       </c>
       <c r="D71" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E71" t="n">
-        <v>13.72473537879843</v>
-      </c>
-      <c r="F71" t="n">
-        <v>73.2208742145525</v>
+        <v>32.8201718685289</v>
       </c>
     </row>
     <row r="72">
@@ -1759,16 +1329,10 @@
         <v>11</v>
       </c>
       <c r="C72" t="n">
-        <v>0</v>
+        <v>23.59714088969098</v>
       </c>
       <c r="D72" t="n">
-        <v>0</v>
-      </c>
-      <c r="E72" t="n">
-        <v>0</v>
-      </c>
-      <c r="F72" t="n">
-        <v>0</v>
+        <v>18.16354363922914</v>
       </c>
     </row>
     <row r="73">
@@ -1782,12 +1346,6 @@
       <c r="D73" t="n">
         <v>0</v>
       </c>
-      <c r="E73" t="n">
-        <v>0</v>
-      </c>
-      <c r="F73" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -1797,16 +1355,10 @@
         <v>1</v>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>41.1245999415783</v>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
-      </c>
-      <c r="E74" t="n">
-        <v>0</v>
-      </c>
-      <c r="F74" t="n">
-        <v>0</v>
+        <v>28.97011605536196</v>
       </c>
     </row>
     <row r="75">
@@ -1815,16 +1367,10 @@
         <v>2</v>
       </c>
       <c r="C75" t="n">
-        <v>0</v>
+        <v>12.97006647483353</v>
       </c>
       <c r="D75" t="n">
-        <v>0</v>
-      </c>
-      <c r="E75" t="n">
-        <v>0</v>
-      </c>
-      <c r="F75" t="n">
-        <v>0</v>
+        <v>11.64835778377565</v>
       </c>
     </row>
     <row r="76">
@@ -1833,16 +1379,10 @@
         <v>3</v>
       </c>
       <c r="C76" t="n">
-        <v>43.16222943024525</v>
+        <v>7.80093670530111</v>
       </c>
       <c r="D76" t="n">
-        <v>159.5582516721107</v>
-      </c>
-      <c r="E76" t="n">
-        <v>94.65742168281739</v>
-      </c>
-      <c r="F76" t="n">
-        <v>128.7444206397463</v>
+        <v>35.30110482966853</v>
       </c>
     </row>
     <row r="77">
@@ -1851,16 +1391,10 @@
         <v>4</v>
       </c>
       <c r="C77" t="n">
-        <v>14.97537512483203</v>
+        <v>73.64115078276802</v>
       </c>
       <c r="D77" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E77" t="n">
-        <v>120.9835134475275</v>
-      </c>
-      <c r="F77" t="n">
-        <v>43.25966343016587</v>
+        <v>167.3222434284612</v>
       </c>
     </row>
     <row r="78">
@@ -1869,16 +1403,10 @@
         <v>5</v>
       </c>
       <c r="C78" t="n">
-        <v>10.98789725807903</v>
+        <v>26.42223684799714</v>
       </c>
       <c r="D78" t="n">
-        <v>31.91165033442215</v>
-      </c>
-      <c r="E78" t="n">
-        <v>77.80818395668631</v>
-      </c>
-      <c r="F78" t="n">
-        <v>37.91799306030711</v>
+        <v>13.36546359751518</v>
       </c>
     </row>
     <row r="79">
@@ -1887,16 +1415,10 @@
         <v>6</v>
       </c>
       <c r="C79" t="n">
-        <v>10.88752420413634</v>
+        <v>49.81956766583758</v>
       </c>
       <c r="D79" t="n">
-        <v>31.91165033442215</v>
-      </c>
-      <c r="E79" t="n">
-        <v>77.09741602156343</v>
-      </c>
-      <c r="F79" t="n">
-        <v>37.91799306030709</v>
+        <v>25.80274963058567</v>
       </c>
     </row>
     <row r="80">
@@ -1905,16 +1427,10 @@
         <v>7</v>
       </c>
       <c r="C80" t="n">
-        <v>9.778804316552959</v>
+        <v>23.51477063113259</v>
       </c>
       <c r="D80" t="n">
-        <v>31.91165033442215</v>
-      </c>
-      <c r="E80" t="n">
-        <v>69.24627954446406</v>
-      </c>
-      <c r="F80" t="n">
-        <v>37.91799306030711</v>
+        <v>13.36546359751518</v>
       </c>
     </row>
     <row r="81">
@@ -1928,12 +1444,6 @@
       <c r="D81" t="n">
         <v>0</v>
       </c>
-      <c r="E81" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n"/>
@@ -1946,12 +1456,6 @@
       <c r="D82" t="n">
         <v>0</v>
       </c>
-      <c r="E82" t="n">
-        <v>0</v>
-      </c>
-      <c r="F82" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n"/>
@@ -1959,16 +1463,10 @@
         <v>10</v>
       </c>
       <c r="C83" t="n">
-        <v>0</v>
+        <v>56.94852571305628</v>
       </c>
       <c r="D83" t="n">
-        <v>0</v>
-      </c>
-      <c r="E83" t="n">
-        <v>0</v>
-      </c>
-      <c r="F83" t="n">
-        <v>0</v>
+        <v>213.6774116811452</v>
       </c>
     </row>
     <row r="84">
@@ -1982,12 +1480,6 @@
       <c r="D84" t="n">
         <v>0</v>
       </c>
-      <c r="E84" t="n">
-        <v>0</v>
-      </c>
-      <c r="F84" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n"/>
@@ -2000,12 +1492,6 @@
       <c r="D85" t="n">
         <v>0</v>
       </c>
-      <c r="E85" t="n">
-        <v>0</v>
-      </c>
-      <c r="F85" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -2015,16 +1501,10 @@
         <v>1</v>
       </c>
       <c r="C86" t="n">
-        <v>15.15458679423914</v>
+        <v>7.800468201887787</v>
       </c>
       <c r="D86" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E86" t="n">
-        <v>34.32557182678543</v>
-      </c>
-      <c r="F86" t="n">
-        <v>12.12853470204306</v>
+        <v>2.860919299920783</v>
       </c>
     </row>
     <row r="87">
@@ -2033,16 +1513,10 @@
         <v>2</v>
       </c>
       <c r="C87" t="n">
-        <v>0</v>
+        <v>27.28206729974161</v>
       </c>
       <c r="D87" t="n">
-        <v>0</v>
-      </c>
-      <c r="E87" t="n">
-        <v>0</v>
-      </c>
-      <c r="F87" t="n">
-        <v>0</v>
+        <v>18.16354363922914</v>
       </c>
     </row>
     <row r="88">
@@ -2051,16 +1525,10 @@
         <v>3</v>
       </c>
       <c r="C88" t="n">
-        <v>0</v>
+        <v>9.633463879408501</v>
       </c>
       <c r="D88" t="n">
-        <v>0</v>
-      </c>
-      <c r="E88" t="n">
-        <v>0</v>
-      </c>
-      <c r="F88" t="n">
-        <v>0</v>
+        <v>11.51392941433848</v>
       </c>
     </row>
     <row r="89">
@@ -2069,16 +1537,10 @@
         <v>4</v>
       </c>
       <c r="C89" t="n">
-        <v>0</v>
+        <v>89.54937197192771</v>
       </c>
       <c r="D89" t="n">
-        <v>0</v>
-      </c>
-      <c r="E89" t="n">
-        <v>0</v>
-      </c>
-      <c r="F89" t="n">
-        <v>0</v>
+        <v>164.1407998103816</v>
       </c>
     </row>
     <row r="90">
@@ -2092,12 +1554,6 @@
       <c r="D90" t="n">
         <v>0</v>
       </c>
-      <c r="E90" t="n">
-        <v>0</v>
-      </c>
-      <c r="F90" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n"/>
@@ -2105,16 +1561,10 @@
         <v>6</v>
       </c>
       <c r="C91" t="n">
-        <v>19.37680829827644</v>
+        <v>31.96532833148086</v>
       </c>
       <c r="D91" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E91" t="n">
-        <v>109.328297420856</v>
-      </c>
-      <c r="F91" t="n">
-        <v>90.63715198172696</v>
+        <v>27.50725273704005</v>
       </c>
     </row>
     <row r="92">
@@ -2128,12 +1578,6 @@
       <c r="D92" t="n">
         <v>0</v>
       </c>
-      <c r="E92" t="n">
-        <v>0</v>
-      </c>
-      <c r="F92" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n"/>
@@ -2146,12 +1590,6 @@
       <c r="D93" t="n">
         <v>0</v>
       </c>
-      <c r="E93" t="n">
-        <v>0</v>
-      </c>
-      <c r="F93" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n"/>
@@ -2164,12 +1602,6 @@
       <c r="D94" t="n">
         <v>0</v>
       </c>
-      <c r="E94" t="n">
-        <v>0</v>
-      </c>
-      <c r="F94" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n"/>
@@ -2177,16 +1609,10 @@
         <v>10</v>
       </c>
       <c r="C95" t="n">
-        <v>6.504552983594778</v>
+        <v>13.4649977515138</v>
       </c>
       <c r="D95" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E95" t="n">
-        <v>36.70014649643929</v>
-      </c>
-      <c r="F95" t="n">
-        <v>30.21238399390899</v>
+        <v>11.64835778377565</v>
       </c>
     </row>
     <row r="96">
@@ -2200,12 +1626,6 @@
       <c r="D96" t="n">
         <v>0</v>
       </c>
-      <c r="E96" t="n">
-        <v>0</v>
-      </c>
-      <c r="F96" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n"/>
@@ -2213,16 +1633,10 @@
         <v>12</v>
       </c>
       <c r="C97" t="n">
-        <v>0</v>
+        <v>18.92685927043278</v>
       </c>
       <c r="D97" t="n">
-        <v>0</v>
-      </c>
-      <c r="E97" t="n">
-        <v>0</v>
-      </c>
-      <c r="F97" t="n">
-        <v>0</v>
+        <v>42.00385914370115</v>
       </c>
     </row>
     <row r="98">
@@ -2236,12 +1650,6 @@
         <v>0</v>
       </c>
       <c r="D98" t="n">
-        <v>0</v>
-      </c>
-      <c r="E98" t="n">
-        <v>0</v>
-      </c>
-      <c r="F98" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2251,16 +1659,10 @@
         <v>2</v>
       </c>
       <c r="C99" t="n">
-        <v>0</v>
+        <v>10.95521144345258</v>
       </c>
       <c r="D99" t="n">
-        <v>0</v>
-      </c>
-      <c r="E99" t="n">
-        <v>0</v>
-      </c>
-      <c r="F99" t="n">
-        <v>0</v>
+        <v>10.93895100748031</v>
       </c>
     </row>
     <row r="100">
@@ -2269,16 +1671,10 @@
         <v>3</v>
       </c>
       <c r="C100" t="n">
-        <v>0</v>
+        <v>31.70196231200855</v>
       </c>
       <c r="D100" t="n">
-        <v>0</v>
-      </c>
-      <c r="E100" t="n">
-        <v>0</v>
-      </c>
-      <c r="F100" t="n">
-        <v>0</v>
+        <v>35.53350409667626</v>
       </c>
     </row>
     <row r="101">
@@ -2292,12 +1688,6 @@
       <c r="D101" t="n">
         <v>0</v>
       </c>
-      <c r="E101" t="n">
-        <v>0</v>
-      </c>
-      <c r="F101" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n"/>
@@ -2305,16 +1695,10 @@
         <v>5</v>
       </c>
       <c r="C102" t="n">
-        <v>8.573166704894742</v>
+        <v>19.87948434822667</v>
       </c>
       <c r="D102" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E102" t="n">
-        <v>61.9733441823685</v>
-      </c>
-      <c r="F102" t="n">
-        <v>110.4363297194324</v>
+        <v>40.23233295885687</v>
       </c>
     </row>
     <row r="103">
@@ -2328,12 +1712,6 @@
       <c r="D103" t="n">
         <v>0</v>
       </c>
-      <c r="E103" t="n">
-        <v>0</v>
-      </c>
-      <c r="F103" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n"/>
@@ -2341,16 +1719,10 @@
         <v>7</v>
       </c>
       <c r="C104" t="n">
-        <v>6.931810654771717</v>
+        <v>11.4351961427592</v>
       </c>
       <c r="D104" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E104" t="n">
-        <v>39.11083008429983</v>
-      </c>
-      <c r="F104" t="n">
-        <v>30.21238399390899</v>
+        <v>9.169084245680017</v>
       </c>
     </row>
     <row r="105">
@@ -2359,16 +1731,10 @@
         <v>8</v>
       </c>
       <c r="C105" t="n">
-        <v>0</v>
+        <v>22.67228868655841</v>
       </c>
       <c r="D105" t="n">
-        <v>0</v>
-      </c>
-      <c r="E105" t="n">
-        <v>0</v>
-      </c>
-      <c r="F105" t="n">
-        <v>0</v>
+        <v>14.91377382815446</v>
       </c>
     </row>
     <row r="106">
@@ -2377,16 +1743,10 @@
         <v>9</v>
       </c>
       <c r="C106" t="n">
-        <v>0</v>
+        <v>7.238329807758571</v>
       </c>
       <c r="D106" t="n">
-        <v>0</v>
-      </c>
-      <c r="E106" t="n">
-        <v>0</v>
-      </c>
-      <c r="F106" t="n">
-        <v>0</v>
+        <v>6.826494886212494</v>
       </c>
     </row>
     <row r="107">
@@ -2395,16 +1755,10 @@
         <v>10</v>
       </c>
       <c r="C107" t="n">
-        <v>0</v>
+        <v>27.3722498582622</v>
       </c>
       <c r="D107" t="n">
-        <v>0</v>
-      </c>
-      <c r="E107" t="n">
-        <v>0</v>
-      </c>
-      <c r="F107" t="n">
-        <v>0</v>
+        <v>13.36546359751518</v>
       </c>
     </row>
     <row r="108">
@@ -2418,12 +1772,6 @@
       <c r="D108" t="n">
         <v>0</v>
       </c>
-      <c r="E108" t="n">
-        <v>0</v>
-      </c>
-      <c r="F108" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n"/>
@@ -2431,16 +1779,10 @@
         <v>12</v>
       </c>
       <c r="C109" t="n">
-        <v>0</v>
+        <v>13.69876048387168</v>
       </c>
       <c r="D109" t="n">
-        <v>0</v>
-      </c>
-      <c r="E109" t="n">
-        <v>0</v>
-      </c>
-      <c r="F109" t="n">
-        <v>0</v>
+        <v>11.51392941433848</v>
       </c>
     </row>
     <row r="110">
@@ -2454,12 +1796,6 @@
         <v>0</v>
       </c>
       <c r="D110" t="n">
-        <v>0</v>
-      </c>
-      <c r="E110" t="n">
-        <v>0</v>
-      </c>
-      <c r="F110" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2469,16 +1805,10 @@
         <v>2</v>
       </c>
       <c r="C111" t="n">
-        <v>12.16917870504368</v>
+        <v>5.428210463098448</v>
       </c>
       <c r="D111" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E111" t="n">
-        <v>0.2486402047273034</v>
-      </c>
-      <c r="F111" t="n">
-        <v>0.1094069067867815</v>
+        <v>2.479273538095631</v>
       </c>
     </row>
     <row r="112">
@@ -2487,16 +1817,10 @@
         <v>3</v>
       </c>
       <c r="C112" t="n">
-        <v>0</v>
+        <v>34.22816888797116</v>
       </c>
       <c r="D112" t="n">
-        <v>0</v>
-      </c>
-      <c r="E112" t="n">
-        <v>0</v>
-      </c>
-      <c r="F112" t="n">
-        <v>0</v>
+        <v>19.60120835628044</v>
       </c>
     </row>
     <row r="113">
@@ -2510,12 +1834,6 @@
       <c r="D113" t="n">
         <v>0</v>
       </c>
-      <c r="E113" t="n">
-        <v>0</v>
-      </c>
-      <c r="F113" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n"/>
@@ -2523,16 +1841,10 @@
         <v>5</v>
       </c>
       <c r="C114" t="n">
-        <v>0</v>
+        <v>47.58091909147388</v>
       </c>
       <c r="D114" t="n">
-        <v>0</v>
-      </c>
-      <c r="E114" t="n">
-        <v>0</v>
-      </c>
-      <c r="F114" t="n">
-        <v>0</v>
+        <v>21.45274253945714</v>
       </c>
     </row>
     <row r="115">
@@ -2541,16 +1853,10 @@
         <v>6</v>
       </c>
       <c r="C115" t="n">
-        <v>7.210563182881756</v>
+        <v>52.11022163514761</v>
       </c>
       <c r="D115" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E115" t="n">
-        <v>12.0186037055473</v>
-      </c>
-      <c r="F115" t="n">
-        <v>8.925231348861518</v>
+        <v>63.82604189770097</v>
       </c>
     </row>
     <row r="116">
@@ -2559,16 +1865,10 @@
         <v>7</v>
       </c>
       <c r="C116" t="n">
-        <v>17.11086327639176</v>
+        <v>22.55672451316866</v>
       </c>
       <c r="D116" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E116" t="n">
-        <v>74.82512076922569</v>
-      </c>
-      <c r="F116" t="n">
-        <v>42.44732860502469</v>
+        <v>12.4372860330705</v>
       </c>
     </row>
     <row r="117">
@@ -2577,16 +1877,10 @@
         <v>8</v>
       </c>
       <c r="C117" t="n">
-        <v>7.933313447101696</v>
+        <v>0</v>
       </c>
       <c r="D117" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E117" t="n">
-        <v>13.22328755387154</v>
-      </c>
-      <c r="F117" t="n">
-        <v>8.925231348861516</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
@@ -2595,16 +1889,10 @@
         <v>9</v>
       </c>
       <c r="C118" t="n">
-        <v>0</v>
+        <v>33.12725539835967</v>
       </c>
       <c r="D118" t="n">
-        <v>0</v>
-      </c>
-      <c r="E118" t="n">
-        <v>0</v>
-      </c>
-      <c r="F118" t="n">
-        <v>0</v>
+        <v>164.3328286484787</v>
       </c>
     </row>
     <row r="119">
@@ -2613,16 +1901,10 @@
         <v>10</v>
       </c>
       <c r="C119" t="n">
-        <v>11.70518922235571</v>
+        <v>55.87471405432665</v>
       </c>
       <c r="D119" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E119" t="n">
-        <v>82.88751658932959</v>
-      </c>
-      <c r="F119" t="n">
-        <v>37.91799306030709</v>
+        <v>31.52900723674432</v>
       </c>
     </row>
     <row r="120">
@@ -2631,16 +1913,10 @@
         <v>11</v>
       </c>
       <c r="C120" t="n">
-        <v>0</v>
+        <v>24.45470133304693</v>
       </c>
       <c r="D120" t="n">
-        <v>0</v>
-      </c>
-      <c r="E120" t="n">
-        <v>0</v>
-      </c>
-      <c r="F120" t="n">
-        <v>0</v>
+        <v>12.4372860330705</v>
       </c>
     </row>
     <row r="121">
@@ -2654,12 +1930,6 @@
       <c r="D121" t="n">
         <v>0</v>
       </c>
-      <c r="E121" t="n">
-        <v>0</v>
-      </c>
-      <c r="F121" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -2669,16 +1939,10 @@
         <v>1</v>
       </c>
       <c r="C122" t="n">
-        <v>0</v>
+        <v>4.931076116276109</v>
       </c>
       <c r="D122" t="n">
-        <v>0</v>
-      </c>
-      <c r="E122" t="n">
-        <v>0</v>
-      </c>
-      <c r="F122" t="n">
-        <v>0</v>
+        <v>2.860919299920783</v>
       </c>
     </row>
     <row r="123">
@@ -2692,12 +1956,6 @@
       <c r="D123" t="n">
         <v>0</v>
       </c>
-      <c r="E123" t="n">
-        <v>0</v>
-      </c>
-      <c r="F123" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n"/>
@@ -2705,16 +1963,10 @@
         <v>3</v>
       </c>
       <c r="C124" t="n">
-        <v>0</v>
+        <v>33.68683651732937</v>
       </c>
       <c r="D124" t="n">
-        <v>0</v>
-      </c>
-      <c r="E124" t="n">
-        <v>0</v>
-      </c>
-      <c r="F124" t="n">
-        <v>0</v>
+        <v>62.1264974263537</v>
       </c>
     </row>
     <row r="125">
@@ -2723,16 +1975,10 @@
         <v>4</v>
       </c>
       <c r="C125" t="n">
-        <v>10.76088020450071</v>
+        <v>49.72783629355434</v>
       </c>
       <c r="D125" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E125" t="n">
-        <v>148.5293282991233</v>
-      </c>
-      <c r="F125" t="n">
-        <v>530.3210734562709</v>
+        <v>162.5596430405904</v>
       </c>
     </row>
     <row r="126">
@@ -2741,16 +1987,10 @@
         <v>5</v>
       </c>
       <c r="C126" t="n">
-        <v>1.963151103952886</v>
+        <v>182.4407305061453</v>
       </c>
       <c r="D126" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E126" t="n">
-        <v>91.67554063590867</v>
-      </c>
-      <c r="F126" t="n">
-        <v>500.108689462362</v>
+        <v>173.9009973808877</v>
       </c>
     </row>
     <row r="127">
@@ -2759,16 +1999,10 @@
         <v>6</v>
       </c>
       <c r="C127" t="n">
-        <v>0</v>
+        <v>33.9270424092587</v>
       </c>
       <c r="D127" t="n">
-        <v>0</v>
-      </c>
-      <c r="E127" t="n">
-        <v>0</v>
-      </c>
-      <c r="F127" t="n">
-        <v>0</v>
+        <v>65.63868431401383</v>
       </c>
     </row>
     <row r="128">
@@ -2777,16 +2011,10 @@
         <v>7</v>
       </c>
       <c r="C128" t="n">
-        <v>0</v>
+        <v>14.1228623834104</v>
       </c>
       <c r="D128" t="n">
-        <v>0</v>
-      </c>
-      <c r="E128" t="n">
-        <v>0</v>
-      </c>
-      <c r="F128" t="n">
-        <v>0</v>
+        <v>20.24637885483243</v>
       </c>
     </row>
     <row r="129">
@@ -2795,16 +2023,10 @@
         <v>8</v>
       </c>
       <c r="C129" t="n">
-        <v>0</v>
+        <v>4.439081739223436</v>
       </c>
       <c r="D129" t="n">
-        <v>0</v>
-      </c>
-      <c r="E129" t="n">
-        <v>0</v>
-      </c>
-      <c r="F129" t="n">
-        <v>0</v>
+        <v>2.479273538095631</v>
       </c>
     </row>
     <row r="130">
@@ -2813,16 +2035,10 @@
         <v>9</v>
       </c>
       <c r="C130" t="n">
-        <v>0</v>
+        <v>14.70526983074578</v>
       </c>
       <c r="D130" t="n">
-        <v>0</v>
-      </c>
-      <c r="E130" t="n">
-        <v>0</v>
-      </c>
-      <c r="F130" t="n">
-        <v>0</v>
+        <v>9.169084245680017</v>
       </c>
     </row>
     <row r="131">
@@ -2831,16 +2047,10 @@
         <v>10</v>
       </c>
       <c r="C131" t="n">
-        <v>6.311559082282605</v>
+        <v>13.62620396464947</v>
       </c>
       <c r="D131" t="n">
-        <v>127.6466013376886</v>
-      </c>
-      <c r="E131" t="n">
-        <v>10.52013905851192</v>
-      </c>
-      <c r="F131" t="n">
-        <v>35.70092539544607</v>
+        <v>9.169084245680017</v>
       </c>
     </row>
     <row r="132">
@@ -2849,16 +2059,10 @@
         <v>11</v>
       </c>
       <c r="C132" t="n">
-        <v>8.733483855128332</v>
+        <v>54.57977469795511</v>
       </c>
       <c r="D132" t="n">
-        <v>31.91165033442215</v>
-      </c>
-      <c r="E132" t="n">
-        <v>49.27627428293466</v>
-      </c>
-      <c r="F132" t="n">
-        <v>30.21238399390899</v>
+        <v>160.7897762787901</v>
       </c>
     </row>
     <row r="133">
@@ -2867,16 +2071,10 @@
         <v>12</v>
       </c>
       <c r="C133" t="n">
-        <v>0</v>
+        <v>4.840905421027808</v>
       </c>
       <c r="D133" t="n">
-        <v>0</v>
-      </c>
-      <c r="E133" t="n">
-        <v>0</v>
-      </c>
-      <c r="F133" t="n">
-        <v>0</v>
+        <v>2.479273538095631</v>
       </c>
     </row>
     <row r="134">
@@ -2887,16 +2085,10 @@
         <v>1</v>
       </c>
       <c r="C134" t="n">
-        <v>0</v>
+        <v>16.85050918006267</v>
       </c>
       <c r="D134" t="n">
-        <v>0</v>
-      </c>
-      <c r="E134" t="n">
-        <v>0</v>
-      </c>
-      <c r="F134" t="n">
-        <v>0</v>
+        <v>17.26000319365749</v>
       </c>
     </row>
     <row r="135">
@@ -2905,16 +2097,10 @@
         <v>2</v>
       </c>
       <c r="C135" t="n">
-        <v>0</v>
+        <v>25.20868786016275</v>
       </c>
       <c r="D135" t="n">
-        <v>0</v>
-      </c>
-      <c r="E135" t="n">
-        <v>0</v>
-      </c>
-      <c r="F135" t="n">
-        <v>0</v>
+        <v>37.88974359938934</v>
       </c>
     </row>
     <row r="136">
@@ -2923,16 +2109,10 @@
         <v>3</v>
       </c>
       <c r="C136" t="n">
-        <v>55.46080988293175</v>
+        <v>165.4295425464529</v>
       </c>
       <c r="D136" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E136" t="n">
-        <v>290.7757997654507</v>
-      </c>
-      <c r="F136" t="n">
-        <v>84.2224673287986</v>
+        <v>49.73672126473598</v>
       </c>
     </row>
     <row r="137">
@@ -2946,12 +2126,6 @@
       <c r="D137" t="n">
         <v>0</v>
       </c>
-      <c r="E137" t="n">
-        <v>0</v>
-      </c>
-      <c r="F137" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n"/>
@@ -2959,16 +2133,10 @@
         <v>5</v>
       </c>
       <c r="C138" t="n">
-        <v>13.4402000031314</v>
+        <v>74.82859732112658</v>
       </c>
       <c r="D138" t="n">
-        <v>191.4699020065329</v>
-      </c>
-      <c r="E138" t="n">
-        <v>92.14349378291431</v>
-      </c>
-      <c r="F138" t="n">
-        <v>168.1205682476638</v>
+        <v>79.86428653345567</v>
       </c>
     </row>
     <row r="139">
@@ -2977,16 +2145,10 @@
         <v>6</v>
       </c>
       <c r="C139" t="n">
-        <v>88.83337105292156</v>
+        <v>136.729930863083</v>
       </c>
       <c r="D139" t="n">
-        <v>414.8514543474878</v>
-      </c>
-      <c r="E139" t="n">
-        <v>217.4659395949224</v>
-      </c>
-      <c r="F139" t="n">
-        <v>206.3751558215031</v>
+        <v>237.581200433221</v>
       </c>
     </row>
     <row r="140">
@@ -2995,16 +2157,10 @@
         <v>7</v>
       </c>
       <c r="C140" t="n">
-        <v>0</v>
+        <v>61.395200265397</v>
       </c>
       <c r="D140" t="n">
-        <v>0</v>
-      </c>
-      <c r="E140" t="n">
-        <v>0</v>
-      </c>
-      <c r="F140" t="n">
-        <v>0</v>
+        <v>39.66904712674705</v>
       </c>
     </row>
     <row r="141">
@@ -3013,16 +2169,10 @@
         <v>8</v>
       </c>
       <c r="C141" t="n">
-        <v>4.41816017093278</v>
+        <v>19.39759498713662</v>
       </c>
       <c r="D141" t="n">
-        <v>31.91165033442215</v>
-      </c>
-      <c r="E141" t="n">
-        <v>15.21018714190514</v>
-      </c>
-      <c r="F141" t="n">
-        <v>18.43434686224036</v>
+        <v>35.53421063347358</v>
       </c>
     </row>
     <row r="142">
@@ -3031,16 +2181,10 @@
         <v>9</v>
       </c>
       <c r="C142" t="n">
-        <v>0</v>
+        <v>16.91392507482635</v>
       </c>
       <c r="D142" t="n">
-        <v>0</v>
-      </c>
-      <c r="E142" t="n">
-        <v>0</v>
-      </c>
-      <c r="F142" t="n">
-        <v>0</v>
+        <v>17.26000319365749</v>
       </c>
     </row>
     <row r="143">
@@ -3049,16 +2193,10 @@
         <v>10</v>
       </c>
       <c r="C143" t="n">
-        <v>0</v>
+        <v>16.50463503177419</v>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
-      </c>
-      <c r="E143" t="n">
-        <v>0</v>
-      </c>
-      <c r="F143" t="n">
-        <v>0</v>
+        <v>31.06324871317685</v>
       </c>
     </row>
     <row r="144">
@@ -3067,16 +2205,10 @@
         <v>11</v>
       </c>
       <c r="C144" t="n">
-        <v>0</v>
+        <v>33.45467972096981</v>
       </c>
       <c r="D144" t="n">
-        <v>0</v>
-      </c>
-      <c r="E144" t="n">
-        <v>0</v>
-      </c>
-      <c r="F144" t="n">
-        <v>0</v>
+        <v>16.22638289743596</v>
       </c>
     </row>
     <row r="145">
@@ -3090,12 +2222,6 @@
       <c r="D145" t="n">
         <v>0</v>
       </c>
-      <c r="E145" t="n">
-        <v>0</v>
-      </c>
-      <c r="F145" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
@@ -3105,16 +2231,10 @@
         <v>1</v>
       </c>
       <c r="C146" t="n">
-        <v>24.16420100643737</v>
+        <v>17.66927346854226</v>
       </c>
       <c r="D146" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E146" t="n">
-        <v>54.7326052861206</v>
-      </c>
-      <c r="F146" t="n">
-        <v>24.25706940408612</v>
+        <v>12.54833348605406</v>
       </c>
     </row>
     <row r="147">
@@ -3123,16 +2243,10 @@
         <v>2</v>
       </c>
       <c r="C147" t="n">
-        <v>0</v>
+        <v>15.58133170713682</v>
       </c>
       <c r="D147" t="n">
-        <v>0</v>
-      </c>
-      <c r="E147" t="n">
-        <v>0</v>
-      </c>
-      <c r="F147" t="n">
-        <v>0</v>
+        <v>71.22580389371504</v>
       </c>
     </row>
     <row r="148">
@@ -3141,16 +2255,10 @@
         <v>3</v>
       </c>
       <c r="C148" t="n">
-        <v>0</v>
+        <v>3.772157281072496</v>
       </c>
       <c r="D148" t="n">
-        <v>0</v>
-      </c>
-      <c r="E148" t="n">
-        <v>0</v>
-      </c>
-      <c r="F148" t="n">
-        <v>0</v>
+        <v>10.9406104305243</v>
       </c>
     </row>
     <row r="149">
@@ -3159,16 +2267,10 @@
         <v>4</v>
       </c>
       <c r="C149" t="n">
-        <v>8.286986725520546</v>
+        <v>50.78798165267477</v>
       </c>
       <c r="D149" t="n">
-        <v>127.6466013376886</v>
-      </c>
-      <c r="E149" t="n">
-        <v>13.81279198878851</v>
-      </c>
-      <c r="F149" t="n">
-        <v>35.70092539544607</v>
+        <v>72.9168521097836</v>
       </c>
     </row>
     <row r="150">
@@ -3177,16 +2279,10 @@
         <v>5</v>
       </c>
       <c r="C150" t="n">
-        <v>7.319972017304093</v>
+        <v>75.21488842804288</v>
       </c>
       <c r="D150" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E150" t="n">
-        <v>145.1778141890491</v>
-      </c>
-      <c r="F150" t="n">
-        <v>106.2002370548432</v>
+        <v>53.69704773590538</v>
       </c>
     </row>
     <row r="151">
@@ -3195,16 +2291,10 @@
         <v>6</v>
       </c>
       <c r="C151" t="n">
-        <v>0</v>
+        <v>23.86171356220115</v>
       </c>
       <c r="D151" t="n">
-        <v>0</v>
-      </c>
-      <c r="E151" t="n">
-        <v>0</v>
-      </c>
-      <c r="F151" t="n">
-        <v>0</v>
+        <v>18.47485266998814</v>
       </c>
     </row>
     <row r="152">
@@ -3213,16 +2303,10 @@
         <v>7</v>
       </c>
       <c r="C152" t="n">
-        <v>14.45958313673779</v>
+        <v>50.70368594162364</v>
       </c>
       <c r="D152" t="n">
-        <v>127.6466013376886</v>
-      </c>
-      <c r="E152" t="n">
-        <v>167.3039612299462</v>
-      </c>
-      <c r="F152" t="n">
-        <v>750.2724411003295</v>
+        <v>216.1566852192408</v>
       </c>
     </row>
     <row r="153">
@@ -3231,16 +2315,10 @@
         <v>8</v>
       </c>
       <c r="C153" t="n">
-        <v>20.98676620077886</v>
+        <v>46.14215021770806</v>
       </c>
       <c r="D153" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E153" t="n">
-        <v>92.29375692649027</v>
-      </c>
-      <c r="F153" t="n">
-        <v>53.21721332143071</v>
+        <v>57.62902033114246</v>
       </c>
     </row>
     <row r="154">
@@ -3249,16 +2327,10 @@
         <v>9</v>
       </c>
       <c r="C154" t="n">
-        <v>19.09985159195995</v>
+        <v>47.56389486199799</v>
       </c>
       <c r="D154" t="n">
-        <v>159.5582516721107</v>
-      </c>
-      <c r="E154" t="n">
-        <v>13.24136580992545</v>
-      </c>
-      <c r="F154" t="n">
-        <v>35.81033230223286</v>
+        <v>38.01277763477188</v>
       </c>
     </row>
     <row r="155">
@@ -3267,16 +2339,10 @@
         <v>10</v>
       </c>
       <c r="C155" t="n">
-        <v>14.94224376393638</v>
+        <v>72.79847540498726</v>
       </c>
       <c r="D155" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E155" t="n">
-        <v>93.54322642039295</v>
-      </c>
-      <c r="F155" t="n">
-        <v>33.52209725616318</v>
+        <v>42.42606811739712</v>
       </c>
     </row>
     <row r="156">
@@ -3285,16 +2351,10 @@
         <v>11</v>
       </c>
       <c r="C156" t="n">
-        <v>0</v>
+        <v>31.13003165795622</v>
       </c>
       <c r="D156" t="n">
-        <v>0</v>
-      </c>
-      <c r="E156" t="n">
-        <v>0</v>
-      </c>
-      <c r="F156" t="n">
-        <v>0</v>
+        <v>18.16354363922914</v>
       </c>
     </row>
     <row r="157">
@@ -3303,16 +2363,10 @@
         <v>12</v>
       </c>
       <c r="C157" t="n">
-        <v>0</v>
+        <v>67.04846671591856</v>
       </c>
       <c r="D157" t="n">
-        <v>0</v>
-      </c>
-      <c r="E157" t="n">
-        <v>0</v>
-      </c>
-      <c r="F157" t="n">
-        <v>0</v>
+        <v>25.74799133392534</v>
       </c>
     </row>
     <row r="158">
@@ -3323,16 +2377,10 @@
         <v>1</v>
       </c>
       <c r="C158" t="n">
-        <v>15.53380745673218</v>
+        <v>130.054111396106</v>
       </c>
       <c r="D158" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E158" t="n">
-        <v>142.6882448869304</v>
-      </c>
-      <c r="F158" t="n">
-        <v>512.237224164405</v>
+        <v>230.8559867167859</v>
       </c>
     </row>
     <row r="159">
@@ -3341,16 +2389,10 @@
         <v>2</v>
       </c>
       <c r="C159" t="n">
-        <v>45.20357040892306</v>
+        <v>223.7671039496106</v>
       </c>
       <c r="D159" t="n">
-        <v>255.2932026753772</v>
-      </c>
-      <c r="E159" t="n">
-        <v>296.4382838868566</v>
-      </c>
-      <c r="F159" t="n">
-        <v>235.7944056252055</v>
+        <v>311.0132747994817</v>
       </c>
     </row>
     <row r="160">
@@ -3359,16 +2401,10 @@
         <v>3</v>
       </c>
       <c r="C160" t="n">
-        <v>8.69227050360263</v>
+        <v>182.4518648266455</v>
       </c>
       <c r="D160" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E160" t="n">
-        <v>49.04373931205851</v>
-      </c>
-      <c r="F160" t="n">
-        <v>30.21238399390899</v>
+        <v>319.4371100733703</v>
       </c>
     </row>
     <row r="161">
@@ -3377,16 +2413,10 @@
         <v>4</v>
       </c>
       <c r="C161" t="n">
-        <v>62.98650281492476</v>
+        <v>279.4072492769962</v>
       </c>
       <c r="D161" t="n">
-        <v>255.2932026753772</v>
-      </c>
-      <c r="E161" t="n">
-        <v>342.1046326521679</v>
-      </c>
-      <c r="F161" t="n">
-        <v>661.8428180991558</v>
+        <v>452.6846546527826</v>
       </c>
     </row>
     <row r="162">
@@ -3395,16 +2425,10 @@
         <v>5</v>
       </c>
       <c r="C162" t="n">
-        <v>15.63523856464719</v>
+        <v>168.3908888337431</v>
       </c>
       <c r="D162" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E162" t="n">
-        <v>90.41036428128118</v>
-      </c>
-      <c r="F162" t="n">
-        <v>117.0926394500041</v>
+        <v>296.1860670956371</v>
       </c>
     </row>
     <row r="163">
@@ -3413,16 +2437,10 @@
         <v>6</v>
       </c>
       <c r="C163" t="n">
-        <v>50.00966346091195</v>
+        <v>88.73166381978388</v>
       </c>
       <c r="D163" t="n">
-        <v>127.6466013376886</v>
-      </c>
-      <c r="E163" t="n">
-        <v>106.2476342783201</v>
-      </c>
-      <c r="F163" t="n">
-        <v>60.64358180139154</v>
+        <v>74.45671535048422</v>
       </c>
     </row>
     <row r="164">
@@ -3431,16 +2449,10 @@
         <v>7</v>
       </c>
       <c r="C164" t="n">
-        <v>0</v>
+        <v>27.03704045500077</v>
       </c>
       <c r="D164" t="n">
-        <v>0</v>
-      </c>
-      <c r="E164" t="n">
-        <v>0</v>
-      </c>
-      <c r="F164" t="n">
-        <v>0</v>
+        <v>18.47485266998814</v>
       </c>
     </row>
     <row r="165">
@@ -3449,16 +2461,10 @@
         <v>8</v>
       </c>
       <c r="C165" t="n">
-        <v>0</v>
+        <v>72.18604300256146</v>
       </c>
       <c r="D165" t="n">
-        <v>0</v>
-      </c>
-      <c r="E165" t="n">
-        <v>0</v>
-      </c>
-      <c r="F165" t="n">
-        <v>0</v>
+        <v>32.62924451679817</v>
       </c>
     </row>
     <row r="166">
@@ -3467,16 +2473,10 @@
         <v>9</v>
       </c>
       <c r="C166" t="n">
-        <v>0</v>
+        <v>54.69657446366934</v>
       </c>
       <c r="D166" t="n">
-        <v>0</v>
-      </c>
-      <c r="E166" t="n">
-        <v>0</v>
-      </c>
-      <c r="F166" t="n">
-        <v>0</v>
+        <v>8.087278941941969</v>
       </c>
     </row>
     <row r="167">
@@ -3485,16 +2485,10 @@
         <v>10</v>
       </c>
       <c r="C167" t="n">
-        <v>0</v>
+        <v>95.76412734111437</v>
       </c>
       <c r="D167" t="n">
-        <v>0</v>
-      </c>
-      <c r="E167" t="n">
-        <v>0</v>
-      </c>
-      <c r="F167" t="n">
-        <v>0</v>
+        <v>108.7351215874265</v>
       </c>
     </row>
     <row r="168">
@@ -3503,16 +2497,10 @@
         <v>11</v>
       </c>
       <c r="C168" t="n">
-        <v>4.10404750737244</v>
+        <v>238.1094363975246</v>
       </c>
       <c r="D168" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E168" t="n">
-        <v>92.01977902285468</v>
-      </c>
-      <c r="F168" t="n">
-        <v>120.0614157683129</v>
+        <v>234.3416436900954</v>
       </c>
     </row>
     <row r="169">
@@ -3521,16 +2509,10 @@
         <v>12</v>
       </c>
       <c r="C169" t="n">
-        <v>52.30477884086506</v>
+        <v>366.8109803589832</v>
       </c>
       <c r="D169" t="n">
-        <v>223.3815523409551</v>
-      </c>
-      <c r="E169" t="n">
-        <v>322.1007704483513</v>
-      </c>
-      <c r="F169" t="n">
-        <v>155.8529263224164</v>
+        <v>138.6683240608168</v>
       </c>
     </row>
     <row r="170">
@@ -3541,16 +2523,10 @@
         <v>1</v>
       </c>
       <c r="C170" t="n">
-        <v>0</v>
+        <v>138.5250234574885</v>
       </c>
       <c r="D170" t="n">
-        <v>0</v>
-      </c>
-      <c r="E170" t="n">
-        <v>0</v>
-      </c>
-      <c r="F170" t="n">
-        <v>0</v>
+        <v>155.5890175506625</v>
       </c>
     </row>
     <row r="171">
@@ -3559,16 +2535,10 @@
         <v>2</v>
       </c>
       <c r="C171" t="n">
-        <v>0</v>
+        <v>19.18354178476588</v>
       </c>
       <c r="D171" t="n">
-        <v>0</v>
-      </c>
-      <c r="E171" t="n">
-        <v>0</v>
-      </c>
-      <c r="F171" t="n">
-        <v>0</v>
+        <v>39.6483261777854</v>
       </c>
     </row>
     <row r="172">
@@ -3577,16 +2547,10 @@
         <v>3</v>
       </c>
       <c r="C172" t="n">
-        <v>9.878928592831658</v>
+        <v>138.3690050115393</v>
       </c>
       <c r="D172" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E172" t="n">
-        <v>0.2018458999858412</v>
-      </c>
-      <c r="F172" t="n">
-        <v>0.1094069067867815</v>
+        <v>337.7907722063459</v>
       </c>
     </row>
     <row r="173">
@@ -3595,16 +2559,10 @@
         <v>4</v>
       </c>
       <c r="C173" t="n">
-        <v>9.251909837396225</v>
+        <v>146.5056351425879</v>
       </c>
       <c r="D173" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E173" t="n">
-        <v>52.20134992530063</v>
-      </c>
-      <c r="F173" t="n">
-        <v>30.21238399390899</v>
+        <v>68.54384652597561</v>
       </c>
     </row>
     <row r="174">
@@ -3613,16 +2571,10 @@
         <v>5</v>
       </c>
       <c r="C174" t="n">
-        <v>9.176486659373973</v>
+        <v>238.5826328562362</v>
       </c>
       <c r="D174" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E174" t="n">
-        <v>91.01231209902728</v>
-      </c>
-      <c r="F174" t="n">
-        <v>53.10780641464392</v>
+        <v>115.9492205737614</v>
       </c>
     </row>
     <row r="175">
@@ -3631,16 +2583,10 @@
         <v>6</v>
       </c>
       <c r="C175" t="n">
-        <v>40.45948169564444</v>
+        <v>127.4696539008041</v>
       </c>
       <c r="D175" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E175" t="n">
-        <v>241.6278173388439</v>
-      </c>
-      <c r="F175" t="n">
-        <v>42.22000819489467</v>
+        <v>85.3644174278279</v>
       </c>
     </row>
     <row r="176">
@@ -3649,16 +2595,10 @@
         <v>7</v>
       </c>
       <c r="C176" t="n">
-        <v>12.43811083112199</v>
+        <v>266.311292779793</v>
       </c>
       <c r="D176" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E176" t="n">
-        <v>28.17267620160352</v>
-      </c>
-      <c r="F176" t="n">
-        <v>12.12853470204306</v>
+        <v>229.3232959644335</v>
       </c>
     </row>
     <row r="177">
@@ -3667,16 +2607,10 @@
         <v>8</v>
       </c>
       <c r="C177" t="n">
-        <v>12.52990341857976</v>
+        <v>214.3660754492314</v>
       </c>
       <c r="D177" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E177" t="n">
-        <v>161.9999077456899</v>
-      </c>
-      <c r="F177" t="n">
-        <v>173.1692221829569</v>
+        <v>332.3302607126742</v>
       </c>
     </row>
     <row r="178">
@@ -3685,16 +2619,10 @@
         <v>9</v>
       </c>
       <c r="C178" t="n">
-        <v>4.40184282943683</v>
+        <v>41.61050863877016</v>
       </c>
       <c r="D178" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E178" t="n">
-        <v>15.15401221654941</v>
-      </c>
-      <c r="F178" t="n">
-        <v>18.43434686224036</v>
+        <v>32.65636873921438</v>
       </c>
     </row>
     <row r="179">
@@ -3703,16 +2631,10 @@
         <v>10</v>
       </c>
       <c r="C179" t="n">
-        <v>0</v>
+        <v>86.56085900738998</v>
       </c>
       <c r="D179" t="n">
-        <v>0</v>
-      </c>
-      <c r="E179" t="n">
-        <v>0</v>
-      </c>
-      <c r="F179" t="n">
-        <v>0</v>
+        <v>35.39931165340919</v>
       </c>
     </row>
     <row r="180">
@@ -3721,16 +2643,10 @@
         <v>11</v>
       </c>
       <c r="C180" t="n">
-        <v>51.65898956526598</v>
+        <v>154.5419536232181</v>
       </c>
       <c r="D180" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E180" t="n">
-        <v>78.76703332151445</v>
-      </c>
-      <c r="F180" t="n">
-        <v>10.09728487584283</v>
+        <v>110.401857185292</v>
       </c>
     </row>
     <row r="181">
@@ -3739,16 +2655,10 @@
         <v>12</v>
       </c>
       <c r="C181" t="n">
-        <v>0</v>
+        <v>81.39143276740769</v>
       </c>
       <c r="D181" t="n">
-        <v>0</v>
-      </c>
-      <c r="E181" t="n">
-        <v>0</v>
-      </c>
-      <c r="F181" t="n">
-        <v>0</v>
+        <v>56.21390544740409</v>
       </c>
     </row>
     <row r="182">
@@ -3759,16 +2669,10 @@
         <v>1</v>
       </c>
       <c r="C182" t="n">
-        <v>50.85700237634305</v>
+        <v>282.8091922157575</v>
       </c>
       <c r="D182" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E182" t="n">
-        <v>396.4437918214293</v>
-      </c>
-      <c r="F182" t="n">
-        <v>357.4175222988516</v>
+        <v>234.382968184846</v>
       </c>
     </row>
     <row r="183">
@@ -3777,16 +2681,10 @@
         <v>2</v>
       </c>
       <c r="C183" t="n">
-        <v>15.25242204021256</v>
+        <v>223.694548747105</v>
       </c>
       <c r="D183" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E183" t="n">
-        <v>134.3515714109756</v>
-      </c>
-      <c r="F183" t="n">
-        <v>126.3286806291964</v>
+        <v>87.16670922016313</v>
       </c>
     </row>
     <row r="184">
@@ -3795,16 +2693,10 @@
         <v>3</v>
       </c>
       <c r="C184" t="n">
-        <v>4.38659505172066</v>
+        <v>221.82924329302</v>
       </c>
       <c r="D184" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E184" t="n">
-        <v>129.9377074826757</v>
-      </c>
-      <c r="F184" t="n">
-        <v>158.6142892321014</v>
+        <v>228.4716575834568</v>
       </c>
     </row>
     <row r="185">
@@ -3813,16 +2705,10 @@
         <v>4</v>
       </c>
       <c r="C185" t="n">
-        <v>43.10996285935688</v>
+        <v>208.2656198553328</v>
       </c>
       <c r="D185" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E185" t="n">
-        <v>80.41114062197148</v>
-      </c>
-      <c r="F185" t="n">
-        <v>9.987877969056045</v>
+        <v>424.8897552541068</v>
       </c>
     </row>
     <row r="186">
@@ -3831,16 +2717,10 @@
         <v>5</v>
       </c>
       <c r="C186" t="n">
-        <v>1.487641890154018</v>
+        <v>97.28438650698861</v>
       </c>
       <c r="D186" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E186" t="n">
-        <v>69.47013618966324</v>
-      </c>
-      <c r="F186" t="n">
-        <v>250.0543447311809</v>
+        <v>94.18341050773667</v>
       </c>
     </row>
     <row r="187">
@@ -3849,16 +2729,10 @@
         <v>6</v>
       </c>
       <c r="C187" t="n">
-        <v>9.912760540067383</v>
+        <v>142.5020815823688</v>
       </c>
       <c r="D187" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E187" t="n">
-        <v>0.2025371530679844</v>
-      </c>
-      <c r="F187" t="n">
-        <v>0.1094069067867815</v>
+        <v>77.94062601913652</v>
       </c>
     </row>
     <row r="188">
@@ -3867,16 +2741,10 @@
         <v>7</v>
       </c>
       <c r="C188" t="n">
-        <v>43.77561594939603</v>
+        <v>249.665978335058</v>
       </c>
       <c r="D188" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E188" t="n">
-        <v>256.5646087342375</v>
-      </c>
-      <c r="F188" t="n">
-        <v>61.59625303242937</v>
+        <v>154.5870773209822</v>
       </c>
     </row>
     <row r="189">
@@ -3885,16 +2753,10 @@
         <v>8</v>
       </c>
       <c r="C189" t="n">
-        <v>0</v>
+        <v>91.56636215191168</v>
       </c>
       <c r="D189" t="n">
-        <v>0</v>
-      </c>
-      <c r="E189" t="n">
-        <v>0</v>
-      </c>
-      <c r="F189" t="n">
-        <v>0</v>
+        <v>71.01181003024752</v>
       </c>
     </row>
     <row r="190">
@@ -3903,16 +2765,10 @@
         <v>9</v>
       </c>
       <c r="C190" t="n">
-        <v>24.47063109166393</v>
+        <v>178.9106802438269</v>
       </c>
       <c r="D190" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E190" t="n">
-        <v>153.1939795000638</v>
-      </c>
-      <c r="F190" t="n">
-        <v>33.52209725616319</v>
+        <v>73.29801033776202</v>
       </c>
     </row>
     <row r="191">
@@ -3921,16 +2777,10 @@
         <v>10</v>
       </c>
       <c r="C191" t="n">
-        <v>32.47064510240021</v>
+        <v>269.3587834658959</v>
       </c>
       <c r="D191" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E191" t="n">
-        <v>354.782679034197</v>
-      </c>
-      <c r="F191" t="n">
-        <v>58.50677309888871</v>
+        <v>200.7827665721997</v>
       </c>
     </row>
     <row r="192">
@@ -3939,16 +2789,10 @@
         <v>11</v>
       </c>
       <c r="C192" t="n">
-        <v>0</v>
+        <v>59.68659206882781</v>
       </c>
       <c r="D192" t="n">
-        <v>0</v>
-      </c>
-      <c r="E192" t="n">
-        <v>0</v>
-      </c>
-      <c r="F192" t="n">
-        <v>0</v>
+        <v>40.98561765733415</v>
       </c>
     </row>
     <row r="193">
@@ -3957,16 +2801,10 @@
         <v>12</v>
       </c>
       <c r="C193" t="n">
-        <v>31.75865177685386</v>
+        <v>312.1049443212432</v>
       </c>
       <c r="D193" t="n">
-        <v>127.6466013376886</v>
-      </c>
-      <c r="E193" t="n">
-        <v>350.4996489243781</v>
-      </c>
-      <c r="F193" t="n">
-        <v>347.6484581433692</v>
+        <v>206.2378981065315</v>
       </c>
     </row>
     <row r="194">
@@ -3977,16 +2815,10 @@
         <v>1</v>
       </c>
       <c r="C194" t="n">
-        <v>5.159583026202631</v>
+        <v>133.4916659724814</v>
       </c>
       <c r="D194" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E194" t="n">
-        <v>35.27644933687343</v>
-      </c>
-      <c r="F194" t="n">
-        <v>73.2208742145525</v>
+        <v>87.69314709957401</v>
       </c>
     </row>
     <row r="195">
@@ -3995,16 +2827,10 @@
         <v>2</v>
       </c>
       <c r="C195" t="n">
-        <v>4.126615589388541</v>
+        <v>5.068305067021176</v>
       </c>
       <c r="D195" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E195" t="n">
-        <v>14.20650065840671</v>
-      </c>
-      <c r="F195" t="n">
-        <v>18.43434686224036</v>
+        <v>6.826494886212494</v>
       </c>
     </row>
     <row r="196">
@@ -4013,16 +2839,10 @@
         <v>3</v>
       </c>
       <c r="C196" t="n">
-        <v>31.98371356574227</v>
+        <v>36.92426037917923</v>
       </c>
       <c r="D196" t="n">
-        <v>63.8233006688443</v>
-      </c>
-      <c r="E196" t="n">
-        <v>72.44402451840904</v>
-      </c>
-      <c r="F196" t="n">
-        <v>24.25706940408613</v>
+        <v>34.42623550101468</v>
       </c>
     </row>
     <row r="197">
@@ -4031,16 +2851,10 @@
         <v>4</v>
       </c>
       <c r="C197" t="n">
-        <v>7.01338959636474</v>
+        <v>53.40536506929195</v>
       </c>
       <c r="D197" t="n">
-        <v>31.91165033442215</v>
-      </c>
-      <c r="E197" t="n">
-        <v>139.0973311440942</v>
-      </c>
-      <c r="F197" t="n">
-        <v>106.2002370548432</v>
+        <v>46.47245510415657</v>
       </c>
     </row>
     <row r="198">
@@ -4049,16 +2863,10 @@
         <v>5</v>
       </c>
       <c r="C198" t="n">
-        <v>10.20739674755553</v>
+        <v>85.12648741219544</v>
       </c>
       <c r="D198" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E198" t="n">
-        <v>57.59242132816544</v>
-      </c>
-      <c r="F198" t="n">
-        <v>30.21238399390899</v>
+        <v>85.07160547984125</v>
       </c>
     </row>
     <row r="199">
@@ -4067,16 +2875,10 @@
         <v>6</v>
       </c>
       <c r="C199" t="n">
-        <v>19.38916989846673</v>
+        <v>8.648775522544419</v>
       </c>
       <c r="D199" t="n">
-        <v>63.82330066884429</v>
-      </c>
-      <c r="E199" t="n">
-        <v>0.3961587950918279</v>
-      </c>
-      <c r="F199" t="n">
-        <v>0.218813813573563</v>
+        <v>4.958547076191262</v>
       </c>
     </row>
     <row r="200">
@@ -4085,16 +2887,10 @@
         <v>7</v>
       </c>
       <c r="C200" t="n">
-        <v>0</v>
+        <v>37.70757563485872</v>
       </c>
       <c r="D200" t="n">
-        <v>0</v>
-      </c>
-      <c r="E200" t="n">
-        <v>0</v>
-      </c>
-      <c r="F200" t="n">
-        <v>0</v>
+        <v>89.83734074233129</v>
       </c>
     </row>
     <row r="201">
@@ -4103,16 +2899,10 @@
         <v>8</v>
       </c>
       <c r="C201" t="n">
-        <v>17.82030126991885</v>
+        <v>109.0902444047529</v>
       </c>
       <c r="D201" t="n">
-        <v>31.91165033442215</v>
-      </c>
-      <c r="E201" t="n">
-        <v>93.43016022953209</v>
-      </c>
-      <c r="F201" t="n">
-        <v>28.0741557762662</v>
+        <v>40.05258783352926</v>
       </c>
     </row>
     <row r="202">
@@ -4121,16 +2911,10 @@
         <v>9</v>
       </c>
       <c r="C202" t="n">
-        <v>40.72760630666451</v>
+        <v>91.84108447473984</v>
       </c>
       <c r="D202" t="n">
-        <v>319.1165033442214</v>
-      </c>
-      <c r="E202" t="n">
-        <v>286.3457847361935</v>
-      </c>
-      <c r="F202" t="n">
-        <v>215.5200809060424</v>
+        <v>59.83791870167174</v>
       </c>
     </row>
     <row r="203">
@@ -4139,16 +2923,10 @@
         <v>10</v>
       </c>
       <c r="C203" t="n">
-        <v>31.03763516468029</v>
+        <v>27.72924911001008</v>
       </c>
       <c r="D203" t="n">
-        <v>223.381552340955</v>
-      </c>
-      <c r="E203" t="n">
-        <v>43.83158041377807</v>
-      </c>
-      <c r="F203" t="n">
-        <v>100.2153820747106</v>
+        <v>48.72098879828846</v>
       </c>
     </row>
     <row r="204">
@@ -4157,16 +2935,10 @@
         <v>11</v>
       </c>
       <c r="C204" t="n">
-        <v>22.38711796090471</v>
+        <v>36.86782180056895</v>
       </c>
       <c r="D204" t="n">
-        <v>95.73495100326643</v>
-      </c>
-      <c r="E204" t="n">
-        <v>18.18285303063616</v>
-      </c>
-      <c r="F204" t="n">
-        <v>36.82925092084981</v>
+        <v>57.90301665041671</v>
       </c>
     </row>
     <row r="205">
@@ -4175,16 +2947,10 @@
         <v>12</v>
       </c>
       <c r="C205" t="n">
-        <v>0</v>
+        <v>60.10621859736482</v>
       </c>
       <c r="D205" t="n">
-        <v>0</v>
-      </c>
-      <c r="E205" t="n">
-        <v>0</v>
-      </c>
-      <c r="F205" t="n">
-        <v>0</v>
+        <v>46.90798584878765</v>
       </c>
     </row>
     <row r="206">
@@ -4195,16 +2961,10 @@
         <v>1</v>
       </c>
       <c r="C206" t="n">
-        <v>10.81776964436611</v>
+        <v>303.309916546203</v>
       </c>
       <c r="D206" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E206" t="n">
-        <v>0.2210282652808116</v>
-      </c>
-      <c r="F206" t="n">
-        <v>0.1094069067867815</v>
+        <v>314.7676310233977</v>
       </c>
     </row>
     <row r="207">
@@ -4213,16 +2973,10 @@
         <v>2</v>
       </c>
       <c r="C207" t="n">
-        <v>3.589950840520505</v>
+        <v>210.5653181342403</v>
       </c>
       <c r="D207" t="n">
-        <v>31.91165033442214</v>
-      </c>
-      <c r="E207" t="n">
-        <v>53.78459049519885</v>
-      </c>
-      <c r="F207" t="n">
-        <v>80.22394572552345</v>
+        <v>195.278272580785</v>
       </c>
     </row>
     <row r="208">
@@ -4231,16 +2985,10 @@
         <v>3</v>
       </c>
       <c r="C208" t="n">
-        <v>9.745879049493858</v>
+        <v>223.9022592502805</v>
       </c>
       <c r="D208" t="n">
-        <v>31.91165033442215</v>
-      </c>
-      <c r="E208" t="n">
-        <v>0.1991274366863685</v>
-      </c>
-      <c r="F208" t="n">
-        <v>0.1094069067867815</v>
+        <v>238.0282084559564</v>
       </c>
     </row>
     <row r="209">
@@ -4249,16 +2997,10 @@
         <v>4</v>
       </c>
       <c r="C209" t="n">
-        <v>225.6288954198081</v>
+        <v>539.9628587258261</v>
       </c>
       <c r="D209" t="n">
-        <v>1021.172810701509</v>
-      </c>
-      <c r="E209" t="n">
-        <v>647.7046942166511</v>
-      </c>
-      <c r="F209" t="n">
-        <v>751.7294267660457</v>
+        <v>665.4885268439618</v>
       </c>
     </row>
     <row r="210">
@@ -4267,16 +3009,10 @@
         <v>5</v>
       </c>
       <c r="C210" t="n">
-        <v>17400.98291092776</v>
+        <v>301.3220593222113</v>
       </c>
       <c r="D210" t="n">
-        <v>638.233006688443</v>
-      </c>
-      <c r="E210" t="n">
-        <v>457.7963930141021</v>
-      </c>
-      <c r="F210" t="n">
-        <v>219.0165538951268</v>
+        <v>293.4372096909116</v>
       </c>
     </row>
     <row r="211">
@@ -4285,16 +3021,10 @@
         <v>6</v>
       </c>
       <c r="C211" t="n">
-        <v>346.89485000502</v>
+        <v>1058.702037133946</v>
       </c>
       <c r="D211" t="n">
-        <v>2010.433971068595</v>
-      </c>
-      <c r="E211" t="n">
-        <v>1570.795396617163</v>
-      </c>
-      <c r="F211" t="n">
-        <v>1748.903391039231</v>
+        <v>1080.911394641637</v>
       </c>
     </row>
     <row r="212">
@@ -4303,16 +3033,10 @@
         <v>7</v>
       </c>
       <c r="C212" t="n">
-        <v>203.8178073091736</v>
+        <v>519.5050613688212</v>
       </c>
       <c r="D212" t="n">
-        <v>1723.229118058796</v>
-      </c>
-      <c r="E212" t="n">
-        <v>704.6585956693822</v>
-      </c>
-      <c r="F212" t="n">
-        <v>953.3100583329996</v>
+        <v>605.93607903236</v>
       </c>
     </row>
     <row r="213">
@@ -4321,16 +3045,10 @@
         <v>8</v>
       </c>
       <c r="C213" t="n">
-        <v>266.5313273404085</v>
+        <v>580.0360790225873</v>
       </c>
       <c r="D213" t="n">
-        <v>1308.377663711308</v>
-      </c>
-      <c r="E213" t="n">
-        <v>1057.564781361923</v>
-      </c>
-      <c r="F213" t="n">
-        <v>767.8229809939719</v>
+        <v>615.4985920135333</v>
       </c>
     </row>
     <row r="214">
@@ -4339,16 +3057,10 @@
         <v>9</v>
       </c>
       <c r="C214" t="n">
-        <v>87.56173029746132</v>
+        <v>273.4741789217958</v>
       </c>
       <c r="D214" t="n">
-        <v>797.7912583605536</v>
-      </c>
-      <c r="E214" t="n">
-        <v>377.6140487802669</v>
-      </c>
-      <c r="F214" t="n">
-        <v>605.2322398599023</v>
+        <v>295.2330055624921</v>
       </c>
     </row>
     <row r="215">
@@ -4357,16 +3069,10 @@
         <v>10</v>
       </c>
       <c r="C215" t="n">
-        <v>261.2521083762744</v>
+        <v>1236.489531813095</v>
       </c>
       <c r="D215" t="n">
-        <v>1340.28931404573</v>
-      </c>
-      <c r="E215" t="n">
-        <v>1203.8983099206</v>
-      </c>
-      <c r="F215" t="n">
-        <v>1223.49980106038</v>
+        <v>1274.319428616542</v>
       </c>
     </row>
     <row r="216">
@@ -4375,16 +3081,10 @@
         <v>11</v>
       </c>
       <c r="C216" t="n">
-        <v>242.5042844627363</v>
+        <v>679.8080610834414</v>
       </c>
       <c r="D216" t="n">
-        <v>1212.642712708042</v>
-      </c>
-      <c r="E216" t="n">
-        <v>626.5979037003767</v>
-      </c>
-      <c r="F216" t="n">
-        <v>693.4960258265399</v>
+        <v>642.6605360744878</v>
       </c>
     </row>
     <row r="217">
@@ -4393,16 +3093,10 @@
         <v>12</v>
       </c>
       <c r="C217" t="n">
-        <v>104.5046552412002</v>
+        <v>510.8143752041662</v>
       </c>
       <c r="D217" t="n">
-        <v>638.2330066884429</v>
-      </c>
-      <c r="E217" t="n">
-        <v>325.7752484340685</v>
-      </c>
-      <c r="F217" t="n">
-        <v>429.355561945589</v>
+        <v>370.204056969939</v>
       </c>
     </row>
     <row r="218">
@@ -4413,16 +3107,10 @@
         <v>1</v>
       </c>
       <c r="C218" t="n">
-        <v>83.09040654753727</v>
+        <v>464.8950456627734</v>
       </c>
       <c r="D218" t="n">
-        <v>414.8514543474878</v>
-      </c>
-      <c r="E218" t="n">
-        <v>588.3170181116585</v>
-      </c>
-      <c r="F218" t="n">
-        <v>494.7283903668313</v>
+        <v>404.8897658632732</v>
       </c>
     </row>
     <row r="219">
@@ -4431,16 +3119,10 @@
         <v>2</v>
       </c>
       <c r="C219" t="n">
-        <v>160.5581831118299</v>
+        <v>627.4926359854262</v>
       </c>
       <c r="D219" t="n">
-        <v>414.851454347488</v>
-      </c>
-      <c r="E219" t="n">
-        <v>414.1787272983792</v>
-      </c>
-      <c r="F219" t="n">
-        <v>298.9708309874198</v>
+        <v>489.8935866563978</v>
       </c>
     </row>
     <row r="220">
@@ -4449,16 +3131,10 @@
         <v>3</v>
       </c>
       <c r="C220" t="n">
-        <v>64.10247888010487</v>
+        <v>985.5116154818029</v>
       </c>
       <c r="D220" t="n">
-        <v>255.2932026753772</v>
-      </c>
-      <c r="E220" t="n">
-        <v>232.439738778977</v>
-      </c>
-      <c r="F220" t="n">
-        <v>176.3711751574199</v>
+        <v>700.8527040648374</v>
       </c>
     </row>
     <row r="221">
@@ -4467,16 +3143,10 @@
         <v>4</v>
       </c>
       <c r="C221" t="n">
-        <v>66.3372766089074</v>
+        <v>280.2039064675896</v>
       </c>
       <c r="D221" t="n">
-        <v>223.381552340955</v>
-      </c>
-      <c r="E221" t="n">
-        <v>339.0553928955807</v>
-      </c>
-      <c r="F221" t="n">
-        <v>198.5034512418783</v>
+        <v>327.8542962271332</v>
       </c>
     </row>
     <row r="222">
@@ -4485,16 +3155,10 @@
         <v>5</v>
       </c>
       <c r="C222" t="n">
-        <v>200.4533063938459</v>
+        <v>681.375769447817</v>
       </c>
       <c r="D222" t="n">
-        <v>670.1446570228651</v>
-      </c>
-      <c r="E222" t="n">
-        <v>713.3840293531545</v>
-      </c>
-      <c r="F222" t="n">
-        <v>624.8207169217885</v>
+        <v>570.4725314266174</v>
       </c>
     </row>
     <row r="223">
@@ -4503,16 +3167,10 @@
         <v>6</v>
       </c>
       <c r="C223" t="n">
-        <v>166.6158099379013</v>
+        <v>403.9691894022718</v>
       </c>
       <c r="D223" t="n">
-        <v>398.8956291802768</v>
-      </c>
-      <c r="E223" t="n">
-        <v>477.0829345504874</v>
-      </c>
-      <c r="F223" t="n">
-        <v>223.7030406350341</v>
+        <v>317.9251592921427</v>
       </c>
     </row>
     <row r="224">
@@ -4521,24 +3179,42 @@
         <v>7</v>
       </c>
       <c r="C224" t="n">
-        <v>151.1557932899051</v>
+        <v>341.1166065130264</v>
       </c>
       <c r="D224" t="n">
-        <v>520.2986467568828</v>
-      </c>
-      <c r="E224" t="n">
-        <v>337.9945260896419</v>
-      </c>
-      <c r="F224" t="n">
-        <v>309.5110488147308</v>
+        <v>399.5376876214065</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="1" t="n"/>
+      <c r="B225" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="C225" t="n">
+        <v>416.4458724439396</v>
+      </c>
+      <c r="D225" t="n">
+        <v>290.2774520416102</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="1" t="n"/>
+      <c r="B226" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="C226" t="n">
+        <v>469.8234273737044</v>
+      </c>
+      <c r="D226" t="n">
+        <v>323.8043958357738</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
     <mergeCell ref="A26:A37"/>
     <mergeCell ref="A2:A13"/>
-    <mergeCell ref="A218:A224"/>
     <mergeCell ref="A62:A73"/>
+    <mergeCell ref="A218:A226"/>
     <mergeCell ref="A122:A133"/>
     <mergeCell ref="A38:A49"/>
     <mergeCell ref="A14:A25"/>

</xml_diff>

<commit_message>
Release v2.0.1: Financial Times totals for 2008-2024 from the ETU index
Same newspaper, listed in Factiva as "Financial Times (Available to Academic Subscribers Only)". The REU search returned no total for these months.
</commit_message>
<xml_diff>
--- a/data/processed/index.xlsx
+++ b/data/processed/index.xlsx
@@ -575,10 +575,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>9.178439125865477</v>
+        <v>8.810393218492433</v>
       </c>
       <c r="D10" t="n">
-        <v>11.51392941433847</v>
+        <v>10.81132791863846</v>
       </c>
     </row>
     <row r="11">
@@ -733,10 +733,10 @@
         <v>10</v>
       </c>
       <c r="C23" t="n">
-        <v>3.454881659426192</v>
+        <v>3.316344481397013</v>
       </c>
       <c r="D23" t="n">
-        <v>2.479273538095631</v>
+        <v>2.327983632327562</v>
       </c>
     </row>
     <row r="24">
@@ -771,10 +771,10 @@
         <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>41.81728610087828</v>
+        <v>40.14045621773356</v>
       </c>
       <c r="D26" t="n">
-        <v>44.35918369906828</v>
+        <v>41.65230338971143</v>
       </c>
     </row>
     <row r="27">
@@ -783,10 +783,10 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>12.24810491948888</v>
+        <v>11.75696859152762</v>
       </c>
       <c r="D27" t="n">
-        <v>9.169084245680017</v>
+        <v>8.609569585359827</v>
       </c>
     </row>
     <row r="28">
@@ -795,10 +795,10 @@
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>8.531097992394884</v>
+        <v>8.189009794342661</v>
       </c>
       <c r="D28" t="n">
-        <v>11.51392941433847</v>
+        <v>10.81132791863846</v>
       </c>
     </row>
     <row r="29">
@@ -807,10 +807,10 @@
         <v>4</v>
       </c>
       <c r="C29" t="n">
-        <v>11.89538647854219</v>
+        <v>11.41839379492669</v>
       </c>
       <c r="D29" t="n">
-        <v>22.45453984486278</v>
+        <v>21.08432184955273</v>
       </c>
     </row>
     <row r="30">
@@ -819,10 +819,10 @@
         <v>5</v>
       </c>
       <c r="C30" t="n">
-        <v>40.74350978635739</v>
+        <v>39.10973722184539</v>
       </c>
       <c r="D30" t="n">
-        <v>22.53454784319519</v>
+        <v>21.159447610269</v>
       </c>
     </row>
     <row r="31">
@@ -831,10 +831,10 @@
         <v>6</v>
       </c>
       <c r="C31" t="n">
-        <v>37.01325577200375</v>
+        <v>35.52906253188644</v>
       </c>
       <c r="D31" t="n">
-        <v>95.96794405468442</v>
+        <v>90.11180071684979</v>
       </c>
     </row>
     <row r="32">
@@ -855,10 +855,10 @@
         <v>8</v>
       </c>
       <c r="C33" t="n">
-        <v>41.56610491801685</v>
+        <v>39.89934714028064</v>
       </c>
       <c r="D33" t="n">
-        <v>32.54532128623082</v>
+        <v>30.55934494480324</v>
       </c>
     </row>
     <row r="34">
@@ -867,10 +867,10 @@
         <v>9</v>
       </c>
       <c r="C34" t="n">
-        <v>122.8793525914728</v>
+        <v>117.9520177579832</v>
       </c>
       <c r="D34" t="n">
-        <v>186.0350167870397</v>
+        <v>174.6828123098802</v>
       </c>
     </row>
     <row r="35">
@@ -879,10 +879,10 @@
         <v>10</v>
       </c>
       <c r="C35" t="n">
-        <v>79.78049106334339</v>
+        <v>76.58137596093685</v>
       </c>
       <c r="D35" t="n">
-        <v>94.67082555776153</v>
+        <v>88.89383481529568</v>
       </c>
     </row>
     <row r="36">
@@ -891,10 +891,10 @@
         <v>11</v>
       </c>
       <c r="C36" t="n">
-        <v>120.797832310949</v>
+        <v>115.9539642859063</v>
       </c>
       <c r="D36" t="n">
-        <v>72.67441095647149</v>
+        <v>68.23968255058537</v>
       </c>
     </row>
     <row r="37">
@@ -903,10 +903,10 @@
         <v>12</v>
       </c>
       <c r="C37" t="n">
-        <v>133.6139612685582</v>
+        <v>128.2561797396475</v>
       </c>
       <c r="D37" t="n">
-        <v>182.9147852679767</v>
+        <v>171.7529831507182</v>
       </c>
     </row>
     <row r="38">
@@ -917,10 +917,10 @@
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>57.0143341332905</v>
+        <v>54.72811835611954</v>
       </c>
       <c r="D38" t="n">
-        <v>62.12628901580505</v>
+        <v>58.33522672820425</v>
       </c>
     </row>
     <row r="39">
@@ -929,10 +929,10 @@
         <v>2</v>
       </c>
       <c r="C39" t="n">
-        <v>28.34374438379606</v>
+        <v>27.20718957561671</v>
       </c>
       <c r="D39" t="n">
-        <v>37.3696978698618</v>
+        <v>35.08932905115726</v>
       </c>
     </row>
     <row r="40">
@@ -941,10 +941,10 @@
         <v>3</v>
       </c>
       <c r="C40" t="n">
-        <v>103.3354514560108</v>
+        <v>99.19180682609181</v>
       </c>
       <c r="D40" t="n">
-        <v>126.3911570090188</v>
+        <v>118.6785323469981</v>
       </c>
     </row>
     <row r="41">
@@ -953,10 +953,10 @@
         <v>4</v>
       </c>
       <c r="C41" t="n">
-        <v>25.77887002476456</v>
+        <v>24.74516402320935</v>
       </c>
       <c r="D41" t="n">
-        <v>16.85412225235489</v>
+        <v>15.82565220732675</v>
       </c>
     </row>
     <row r="42">
@@ -965,10 +965,10 @@
         <v>5</v>
       </c>
       <c r="C42" t="n">
-        <v>67.64628909121681</v>
+        <v>64.93374292649531</v>
       </c>
       <c r="D42" t="n">
-        <v>33.83527027586731</v>
+        <v>31.7705788358074</v>
       </c>
     </row>
     <row r="43">
@@ -977,10 +977,10 @@
         <v>6</v>
       </c>
       <c r="C43" t="n">
-        <v>44.29437038248208</v>
+        <v>42.51821198393726</v>
       </c>
       <c r="D43" t="n">
-        <v>37.1914330116954</v>
+        <v>34.92194224786433</v>
       </c>
     </row>
     <row r="44">
@@ -989,10 +989,10 @@
         <v>7</v>
       </c>
       <c r="C44" t="n">
-        <v>99.51422626170849</v>
+        <v>95.52380880632623</v>
       </c>
       <c r="D44" t="n">
-        <v>227.5726401264791</v>
+        <v>213.6857322274131</v>
       </c>
     </row>
     <row r="45">
@@ -1001,10 +1001,10 @@
         <v>8</v>
       </c>
       <c r="C45" t="n">
-        <v>40.46870780496606</v>
+        <v>38.84595451543124</v>
       </c>
       <c r="D45" t="n">
-        <v>16.17455788388394</v>
+        <v>15.18755612692065</v>
       </c>
     </row>
     <row r="46">
@@ -1013,10 +1013,10 @@
         <v>9</v>
       </c>
       <c r="C46" t="n">
-        <v>9.690567709919769</v>
+        <v>9.301985976484669</v>
       </c>
       <c r="D46" t="n">
-        <v>6.826494886212494</v>
+        <v>6.409929407578543</v>
       </c>
     </row>
     <row r="47">
@@ -1025,10 +1025,10 @@
         <v>10</v>
       </c>
       <c r="C47" t="n">
-        <v>77.64168620845801</v>
+        <v>74.52833496662903</v>
       </c>
       <c r="D47" t="n">
-        <v>64.63323916011262</v>
+        <v>60.68919808849718</v>
       </c>
     </row>
     <row r="48">
@@ -1037,10 +1037,10 @@
         <v>11</v>
       </c>
       <c r="C48" t="n">
-        <v>143.6360183643897</v>
+        <v>137.8763627208286</v>
       </c>
       <c r="D48" t="n">
-        <v>115.2991092537007</v>
+        <v>108.2633420799288</v>
       </c>
     </row>
     <row r="49">
@@ -1049,10 +1049,10 @@
         <v>12</v>
       </c>
       <c r="C49" t="n">
-        <v>45.87797060792168</v>
+        <v>44.03831147968899</v>
       </c>
       <c r="D49" t="n">
-        <v>124.2529948527074</v>
+        <v>116.6708448423033</v>
       </c>
     </row>
     <row r="50">
@@ -1063,10 +1063,10 @@
         <v>1</v>
       </c>
       <c r="C50" t="n">
-        <v>174.8803014392545</v>
+        <v>167.8677823886569</v>
       </c>
       <c r="D50" t="n">
-        <v>78.16210863967638</v>
+        <v>73.39251066307988</v>
       </c>
     </row>
     <row r="51">
@@ -1075,10 +1075,10 @@
         <v>2</v>
       </c>
       <c r="C51" t="n">
-        <v>73.72014661828268</v>
+        <v>70.76404505441887</v>
       </c>
       <c r="D51" t="n">
-        <v>36.74336006110997</v>
+        <v>34.5012115463005</v>
       </c>
     </row>
     <row r="52">
@@ -1087,10 +1087,10 @@
         <v>3</v>
       </c>
       <c r="C52" t="n">
-        <v>195.715557245195</v>
+        <v>187.8675660055586</v>
       </c>
       <c r="D52" t="n">
-        <v>266.703200463893</v>
+        <v>250.4284726267953</v>
       </c>
     </row>
     <row r="53">
@@ -1099,10 +1099,10 @@
         <v>4</v>
       </c>
       <c r="C53" t="n">
-        <v>41.13177211930125</v>
+        <v>39.48243063716966</v>
       </c>
       <c r="D53" t="n">
-        <v>37.78796617910261</v>
+        <v>35.48207384630473</v>
       </c>
     </row>
     <row r="54">
@@ -1111,10 +1111,10 @@
         <v>5</v>
       </c>
       <c r="C54" t="n">
-        <v>44.03333451948032</v>
+        <v>42.26764338881601</v>
       </c>
       <c r="D54" t="n">
-        <v>63.82604189770095</v>
+        <v>59.93125751192112</v>
       </c>
     </row>
     <row r="55">
@@ -1123,10 +1123,10 @@
         <v>6</v>
       </c>
       <c r="C55" t="n">
-        <v>13.89925746049752</v>
+        <v>13.34191162492463</v>
       </c>
       <c r="D55" t="n">
-        <v>10.93895100748031</v>
+        <v>10.27143576896637</v>
       </c>
     </row>
     <row r="56">
@@ -1135,10 +1135,10 @@
         <v>7</v>
       </c>
       <c r="C56" t="n">
-        <v>46.92777665183239</v>
+        <v>45.04602138800428</v>
       </c>
       <c r="D56" t="n">
-        <v>24.87939301185365</v>
+        <v>23.36120594354763</v>
       </c>
     </row>
     <row r="57">
@@ -1147,10 +1147,10 @@
         <v>8</v>
       </c>
       <c r="C57" t="n">
-        <v>57.83548184243602</v>
+        <v>55.51633889218527</v>
       </c>
       <c r="D57" t="n">
-        <v>43.33396340050574</v>
+        <v>40.68964395019805</v>
       </c>
     </row>
     <row r="58">
@@ -1159,10 +1159,10 @@
         <v>9</v>
       </c>
       <c r="C58" t="n">
-        <v>4.2859619507581</v>
+        <v>4.114099313385717</v>
       </c>
       <c r="D58" t="n">
-        <v>21.8812208610486</v>
+        <v>20.54598786182855</v>
       </c>
     </row>
     <row r="59">
@@ -1171,10 +1171,10 @@
         <v>10</v>
       </c>
       <c r="C59" t="n">
-        <v>11.28369557861036</v>
+        <v>10.83123106685611</v>
       </c>
       <c r="D59" t="n">
-        <v>46.24171526019283</v>
+        <v>43.41995935598464</v>
       </c>
     </row>
     <row r="60">
@@ -1183,10 +1183,10 @@
         <v>11</v>
       </c>
       <c r="C60" t="n">
-        <v>10.48465443076698</v>
+        <v>10.06423064186915</v>
       </c>
       <c r="D60" t="n">
-        <v>9.169084245680017</v>
+        <v>8.609569585359827</v>
       </c>
     </row>
     <row r="61">
@@ -1233,10 +1233,10 @@
         <v>3</v>
       </c>
       <c r="C64" t="n">
-        <v>237.6361409433172</v>
+        <v>228.1071776938207</v>
       </c>
       <c r="D64" t="n">
-        <v>261.3877223923998</v>
+        <v>245.4373549633781</v>
       </c>
     </row>
     <row r="65">
@@ -1257,10 +1257,10 @@
         <v>5</v>
       </c>
       <c r="C66" t="n">
-        <v>34.91445766048764</v>
+        <v>33.51442405195399</v>
       </c>
       <c r="D66" t="n">
-        <v>16.57890708824532</v>
+        <v>15.56723118698725</v>
       </c>
     </row>
     <row r="67">
@@ -1317,10 +1317,10 @@
         <v>10</v>
       </c>
       <c r="C71" t="n">
-        <v>18.46262659676481</v>
+        <v>17.72229438285417</v>
       </c>
       <c r="D71" t="n">
-        <v>32.8201718685289</v>
+        <v>30.81742363079491</v>
       </c>
     </row>
     <row r="72">
@@ -1329,10 +1329,10 @@
         <v>11</v>
       </c>
       <c r="C72" t="n">
-        <v>23.59714088969098</v>
+        <v>22.65091996791339</v>
       </c>
       <c r="D72" t="n">
-        <v>18.16354363922914</v>
+        <v>17.05517025348973</v>
       </c>
     </row>
     <row r="73">
@@ -1355,10 +1355,10 @@
         <v>1</v>
       </c>
       <c r="C74" t="n">
-        <v>41.1245999415783</v>
+        <v>39.47554605634872</v>
       </c>
       <c r="D74" t="n">
-        <v>28.97011605536196</v>
+        <v>27.20230542020619</v>
       </c>
     </row>
     <row r="75">
@@ -1367,10 +1367,10 @@
         <v>2</v>
       </c>
       <c r="C75" t="n">
-        <v>12.97006647483353</v>
+        <v>12.4499802358818</v>
       </c>
       <c r="D75" t="n">
-        <v>11.64835778377565</v>
+        <v>10.93755321768739</v>
       </c>
     </row>
     <row r="76">
@@ -1379,10 +1379,10 @@
         <v>3</v>
       </c>
       <c r="C76" t="n">
-        <v>7.80093670530111</v>
+        <v>7.488127218994091</v>
       </c>
       <c r="D76" t="n">
-        <v>35.30110482966853</v>
+        <v>33.14696542507038</v>
       </c>
     </row>
     <row r="77">
@@ -1391,10 +1391,10 @@
         <v>4</v>
       </c>
       <c r="C77" t="n">
-        <v>73.64115078276802</v>
+        <v>70.68821687013138</v>
       </c>
       <c r="D77" t="n">
-        <v>167.3222434284612</v>
+        <v>157.1119273611838</v>
       </c>
     </row>
     <row r="78">
@@ -1403,10 +1403,10 @@
         <v>5</v>
       </c>
       <c r="C78" t="n">
-        <v>26.42223684799714</v>
+        <v>25.36273250284743</v>
       </c>
       <c r="D78" t="n">
-        <v>13.36546359751518</v>
+        <v>12.54987802490918</v>
       </c>
     </row>
     <row r="79">
@@ -1415,10 +1415,10 @@
         <v>6</v>
       </c>
       <c r="C79" t="n">
-        <v>49.81956766583758</v>
+        <v>47.82185457594692</v>
       </c>
       <c r="D79" t="n">
-        <v>25.80274963058567</v>
+        <v>24.22821761538622</v>
       </c>
     </row>
     <row r="80">
@@ -1427,10 +1427,10 @@
         <v>7</v>
       </c>
       <c r="C80" t="n">
-        <v>23.51477063113259</v>
+        <v>22.57185267145302</v>
       </c>
       <c r="D80" t="n">
-        <v>13.36546359751518</v>
+        <v>12.54987802490918</v>
       </c>
     </row>
     <row r="81">
@@ -1463,10 +1463,10 @@
         <v>10</v>
       </c>
       <c r="C83" t="n">
-        <v>56.94852571305628</v>
+        <v>54.66494878541145</v>
       </c>
       <c r="D83" t="n">
-        <v>213.6774116811452</v>
+        <v>200.6384165959815</v>
       </c>
     </row>
     <row r="84">
@@ -1501,10 +1501,10 @@
         <v>1</v>
       </c>
       <c r="C86" t="n">
-        <v>7.800468201887787</v>
+        <v>7.487677502082644</v>
       </c>
       <c r="D86" t="n">
-        <v>2.860919299920783</v>
+        <v>2.686340656360732</v>
       </c>
     </row>
     <row r="87">
@@ -1513,10 +1513,10 @@
         <v>2</v>
       </c>
       <c r="C87" t="n">
-        <v>27.28206729974161</v>
+        <v>26.18808464357848</v>
       </c>
       <c r="D87" t="n">
-        <v>18.16354363922914</v>
+        <v>17.05517025348973</v>
       </c>
     </row>
     <row r="88">
@@ -1525,10 +1525,10 @@
         <v>3</v>
       </c>
       <c r="C88" t="n">
-        <v>9.633463879408501</v>
+        <v>9.247171950462681</v>
       </c>
       <c r="D88" t="n">
-        <v>11.51392941433848</v>
+        <v>10.81132791863846</v>
       </c>
     </row>
     <row r="89">
@@ -1537,10 +1537,10 @@
         <v>4</v>
       </c>
       <c r="C89" t="n">
-        <v>89.54937197192771</v>
+        <v>85.95853485788992</v>
       </c>
       <c r="D89" t="n">
-        <v>164.1407998103816</v>
+        <v>154.1246213797102</v>
       </c>
     </row>
     <row r="90">
@@ -1561,10 +1561,10 @@
         <v>6</v>
       </c>
       <c r="C91" t="n">
-        <v>31.96532833148086</v>
+        <v>30.68355175608435</v>
       </c>
       <c r="D91" t="n">
-        <v>27.50725273704005</v>
+        <v>25.82870875607948</v>
       </c>
     </row>
     <row r="92">
@@ -1609,10 +1609,10 @@
         <v>10</v>
       </c>
       <c r="C95" t="n">
-        <v>13.4649977515138</v>
+        <v>12.92506528072296</v>
       </c>
       <c r="D95" t="n">
-        <v>11.64835778377565</v>
+        <v>10.93755321768739</v>
       </c>
     </row>
     <row r="96">
@@ -1633,10 +1633,10 @@
         <v>12</v>
       </c>
       <c r="C97" t="n">
-        <v>18.92685927043278</v>
+        <v>18.16791180688445</v>
       </c>
       <c r="D97" t="n">
-        <v>42.00385914370115</v>
+        <v>39.44070514149009</v>
       </c>
     </row>
     <row r="98">
@@ -1659,10 +1659,10 @@
         <v>2</v>
       </c>
       <c r="C99" t="n">
-        <v>10.95521144345258</v>
+        <v>10.51591880546944</v>
       </c>
       <c r="D99" t="n">
-        <v>10.93895100748031</v>
+        <v>10.27143576896637</v>
       </c>
     </row>
     <row r="100">
@@ -1671,10 +1671,10 @@
         <v>3</v>
       </c>
       <c r="C100" t="n">
-        <v>31.70196231200855</v>
+        <v>30.43074644135483</v>
       </c>
       <c r="D100" t="n">
-        <v>35.53350409667626</v>
+        <v>33.3651832543844</v>
       </c>
     </row>
     <row r="101">
@@ -1695,10 +1695,10 @@
         <v>5</v>
       </c>
       <c r="C102" t="n">
-        <v>19.87948434822667</v>
+        <v>19.08233760522189</v>
       </c>
       <c r="D102" t="n">
-        <v>40.23233295885687</v>
+        <v>37.77728079593565</v>
       </c>
     </row>
     <row r="103">
@@ -1719,10 +1719,10 @@
         <v>7</v>
       </c>
       <c r="C104" t="n">
-        <v>11.4351961427592</v>
+        <v>10.97665661521685</v>
       </c>
       <c r="D104" t="n">
-        <v>9.169084245680017</v>
+        <v>8.609569585359827</v>
       </c>
     </row>
     <row r="105">
@@ -1731,10 +1731,10 @@
         <v>8</v>
       </c>
       <c r="C105" t="n">
-        <v>22.67228868655841</v>
+        <v>21.763153380714</v>
       </c>
       <c r="D105" t="n">
-        <v>14.91377382815446</v>
+        <v>14.00370747103887</v>
       </c>
     </row>
     <row r="106">
@@ -1743,10 +1743,10 @@
         <v>9</v>
       </c>
       <c r="C106" t="n">
-        <v>7.238329807758571</v>
+        <v>6.948080275629038</v>
       </c>
       <c r="D106" t="n">
-        <v>6.826494886212494</v>
+        <v>6.409929407578543</v>
       </c>
     </row>
     <row r="107">
@@ -1755,10 +1755,10 @@
         <v>10</v>
       </c>
       <c r="C107" t="n">
-        <v>27.3722498582622</v>
+        <v>26.27465097485992</v>
       </c>
       <c r="D107" t="n">
-        <v>13.36546359751518</v>
+        <v>12.54987802490918</v>
       </c>
     </row>
     <row r="108">
@@ -1779,10 +1779,10 @@
         <v>12</v>
       </c>
       <c r="C109" t="n">
-        <v>13.69876048387168</v>
+        <v>13.14945436950585</v>
       </c>
       <c r="D109" t="n">
-        <v>11.51392941433848</v>
+        <v>10.81132791863846</v>
       </c>
     </row>
     <row r="110">
@@ -1805,10 +1805,10 @@
         <v>2</v>
       </c>
       <c r="C111" t="n">
-        <v>5.428210463098448</v>
+        <v>5.210544842843595</v>
       </c>
       <c r="D111" t="n">
-        <v>2.479273538095631</v>
+        <v>2.327983632327562</v>
       </c>
     </row>
     <row r="112">
@@ -1817,10 +1817,10 @@
         <v>3</v>
       </c>
       <c r="C112" t="n">
-        <v>34.22816888797116</v>
+        <v>32.85565474876524</v>
       </c>
       <c r="D112" t="n">
-        <v>19.60120835628044</v>
+        <v>18.40510598209879</v>
       </c>
     </row>
     <row r="113">
@@ -1841,10 +1841,10 @@
         <v>5</v>
       </c>
       <c r="C114" t="n">
-        <v>47.58091909147388</v>
+        <v>45.67297349195304</v>
       </c>
       <c r="D114" t="n">
-        <v>21.45274253945714</v>
+        <v>20.1436560883695</v>
       </c>
     </row>
     <row r="115">
@@ -1853,10 +1853,10 @@
         <v>6</v>
       </c>
       <c r="C115" t="n">
-        <v>52.11022163514761</v>
+        <v>50.02065569238608</v>
       </c>
       <c r="D115" t="n">
-        <v>63.82604189770097</v>
+        <v>59.93125751192113</v>
       </c>
     </row>
     <row r="116">
@@ -1865,10 +1865,10 @@
         <v>7</v>
       </c>
       <c r="C116" t="n">
-        <v>22.55672451316866</v>
+        <v>21.65222321104446</v>
       </c>
       <c r="D116" t="n">
-        <v>12.4372860330705</v>
+        <v>11.67833959047705</v>
       </c>
     </row>
     <row r="117">
@@ -1889,10 +1889,10 @@
         <v>9</v>
       </c>
       <c r="C118" t="n">
-        <v>33.12725539835967</v>
+        <v>31.79888675041506</v>
       </c>
       <c r="D118" t="n">
-        <v>164.3328286484787</v>
+        <v>154.3049322591495</v>
       </c>
     </row>
     <row r="119">
@@ -1901,10 +1901,10 @@
         <v>10</v>
       </c>
       <c r="C119" t="n">
-        <v>55.87471405432665</v>
+        <v>53.63419586258074</v>
       </c>
       <c r="D119" t="n">
-        <v>31.52900723674432</v>
+        <v>29.60504827839891</v>
       </c>
     </row>
     <row r="120">
@@ -1913,10 +1913,10 @@
         <v>11</v>
       </c>
       <c r="C120" t="n">
-        <v>24.45470133304693</v>
+        <v>23.47409312524238</v>
       </c>
       <c r="D120" t="n">
-        <v>12.4372860330705</v>
+        <v>11.67833959047705</v>
       </c>
     </row>
     <row r="121">
@@ -1939,10 +1939,10 @@
         <v>1</v>
       </c>
       <c r="C122" t="n">
-        <v>4.931076116276109</v>
+        <v>4.733345068692431</v>
       </c>
       <c r="D122" t="n">
-        <v>2.860919299920783</v>
+        <v>2.686340656360731</v>
       </c>
     </row>
     <row r="123">
@@ -1963,10 +1963,10 @@
         <v>3</v>
       </c>
       <c r="C124" t="n">
-        <v>33.68683651732937</v>
+        <v>32.33602924579574</v>
       </c>
       <c r="D124" t="n">
-        <v>62.1264974263537</v>
+        <v>58.33542242115164</v>
       </c>
     </row>
     <row r="125">
@@ -1975,10 +1975,10 @@
         <v>4</v>
       </c>
       <c r="C125" t="n">
-        <v>49.72783629355434</v>
+        <v>47.73380153673138</v>
       </c>
       <c r="D125" t="n">
-        <v>162.5596430405904</v>
+        <v>152.6399497516472</v>
       </c>
     </row>
     <row r="126">
@@ -1987,10 +1987,10 @@
         <v>5</v>
       </c>
       <c r="C126" t="n">
-        <v>182.4407305061453</v>
+        <v>175.1250460765661</v>
       </c>
       <c r="D126" t="n">
-        <v>173.9009973808877</v>
+        <v>163.2892334498547</v>
       </c>
     </row>
     <row r="127">
@@ -1999,10 +1999,10 @@
         <v>6</v>
       </c>
       <c r="C127" t="n">
-        <v>33.9270424092587</v>
+        <v>32.56660313012124</v>
       </c>
       <c r="D127" t="n">
-        <v>65.63868431401383</v>
+        <v>61.63328909964192</v>
       </c>
     </row>
     <row r="128">
@@ -2011,10 +2011,10 @@
         <v>7</v>
       </c>
       <c r="C128" t="n">
-        <v>14.1228623834104</v>
+        <v>13.55655022190584</v>
       </c>
       <c r="D128" t="n">
-        <v>20.24637885483243</v>
+        <v>19.01090697082038</v>
       </c>
     </row>
     <row r="129">
@@ -2023,10 +2023,10 @@
         <v>8</v>
       </c>
       <c r="C129" t="n">
-        <v>4.439081739223436</v>
+        <v>4.261079156844099</v>
       </c>
       <c r="D129" t="n">
-        <v>2.479273538095631</v>
+        <v>2.327983632327562</v>
       </c>
     </row>
     <row r="130">
@@ -2035,10 +2035,10 @@
         <v>9</v>
       </c>
       <c r="C130" t="n">
-        <v>14.70526983074578</v>
+        <v>14.11560373351468</v>
       </c>
       <c r="D130" t="n">
-        <v>9.169084245680017</v>
+        <v>8.609569585359827</v>
       </c>
     </row>
     <row r="131">
@@ -2047,10 +2047,10 @@
         <v>10</v>
       </c>
       <c r="C131" t="n">
-        <v>13.62620396464947</v>
+        <v>13.07980729159351</v>
       </c>
       <c r="D131" t="n">
-        <v>9.169084245680017</v>
+        <v>8.609569585359827</v>
       </c>
     </row>
     <row r="132">
@@ -2059,10 +2059,10 @@
         <v>11</v>
       </c>
       <c r="C132" t="n">
-        <v>54.57977469795511</v>
+        <v>52.39118223387086</v>
       </c>
       <c r="D132" t="n">
-        <v>160.7897762787901</v>
+        <v>150.9780835680407</v>
       </c>
     </row>
     <row r="133">
@@ -2071,10 +2071,10 @@
         <v>12</v>
       </c>
       <c r="C133" t="n">
-        <v>4.840905421027808</v>
+        <v>4.646790124978353</v>
       </c>
       <c r="D133" t="n">
-        <v>2.479273538095631</v>
+        <v>2.327983632327562</v>
       </c>
     </row>
     <row r="134">
@@ -2085,10 +2085,10 @@
         <v>1</v>
       </c>
       <c r="C134" t="n">
-        <v>16.85050918006267</v>
+        <v>16.17482120568836</v>
       </c>
       <c r="D134" t="n">
-        <v>17.26000319365749</v>
+        <v>16.20676553488315</v>
       </c>
     </row>
     <row r="135">
@@ -2097,10 +2097,10 @@
         <v>2</v>
       </c>
       <c r="C135" t="n">
-        <v>25.20868786016275</v>
+        <v>24.19784557315215</v>
       </c>
       <c r="D135" t="n">
-        <v>37.88974359938934</v>
+        <v>35.57764061815437</v>
       </c>
     </row>
     <row r="136">
@@ -2109,10 +2109,10 @@
         <v>3</v>
       </c>
       <c r="C136" t="n">
-        <v>165.4295425464529</v>
+        <v>158.7959891439754</v>
       </c>
       <c r="D136" t="n">
-        <v>49.73672126473598</v>
+        <v>46.70169356096175</v>
       </c>
     </row>
     <row r="137">
@@ -2133,10 +2133,10 @@
         <v>5</v>
       </c>
       <c r="C138" t="n">
-        <v>74.82859732112658</v>
+        <v>71.82804803155342</v>
       </c>
       <c r="D138" t="n">
-        <v>79.86428653345567</v>
+        <v>74.99081847992197</v>
       </c>
     </row>
     <row r="139">
@@ -2145,10 +2145,10 @@
         <v>6</v>
       </c>
       <c r="C139" t="n">
-        <v>136.729930863083</v>
+        <v>131.2472021791019</v>
       </c>
       <c r="D139" t="n">
-        <v>237.581200433221</v>
+        <v>223.0835514753672</v>
       </c>
     </row>
     <row r="140">
@@ -2157,10 +2157,10 @@
         <v>7</v>
       </c>
       <c r="C140" t="n">
-        <v>61.395200265397</v>
+        <v>58.93331629142695</v>
       </c>
       <c r="D140" t="n">
-        <v>39.66904712674705</v>
+        <v>37.24836771824398</v>
       </c>
     </row>
     <row r="141">
@@ -2169,10 +2169,10 @@
         <v>8</v>
       </c>
       <c r="C141" t="n">
-        <v>19.39759498713662</v>
+        <v>18.61977150865685</v>
       </c>
       <c r="D141" t="n">
-        <v>35.53421063347358</v>
+        <v>33.36584667698564</v>
       </c>
     </row>
     <row r="142">
@@ -2181,10 +2181,10 @@
         <v>9</v>
       </c>
       <c r="C142" t="n">
-        <v>16.91392507482635</v>
+        <v>16.23569418872052</v>
       </c>
       <c r="D142" t="n">
-        <v>17.26000319365749</v>
+        <v>16.20676553488315</v>
       </c>
     </row>
     <row r="143">
@@ -2193,10 +2193,10 @@
         <v>10</v>
       </c>
       <c r="C143" t="n">
-        <v>16.50463503177419</v>
+        <v>15.84281625269528</v>
       </c>
       <c r="D143" t="n">
-        <v>31.06324871317685</v>
+        <v>29.16771121057583</v>
       </c>
     </row>
     <row r="144">
@@ -2205,10 +2205,10 @@
         <v>11</v>
       </c>
       <c r="C144" t="n">
-        <v>33.45467972096981</v>
+        <v>32.11318169664011</v>
       </c>
       <c r="D144" t="n">
-        <v>16.22638289743596</v>
+        <v>15.23621868126991</v>
       </c>
     </row>
     <row r="145">
@@ -2231,10 +2231,10 @@
         <v>1</v>
       </c>
       <c r="C146" t="n">
-        <v>17.66927346854226</v>
+        <v>16.96075389378952</v>
       </c>
       <c r="D146" t="n">
-        <v>12.54833348605406</v>
+        <v>11.78261072030001</v>
       </c>
     </row>
     <row r="147">
@@ -2243,10 +2243,10 @@
         <v>2</v>
       </c>
       <c r="C147" t="n">
-        <v>15.58133170713682</v>
+        <v>14.95653643556685</v>
       </c>
       <c r="D147" t="n">
-        <v>71.22580389371504</v>
+        <v>66.87947219866051</v>
       </c>
     </row>
     <row r="148">
@@ -2255,10 +2255,10 @@
         <v>3</v>
       </c>
       <c r="C148" t="n">
-        <v>3.772157281072496</v>
+        <v>3.62089767906089</v>
       </c>
       <c r="D148" t="n">
-        <v>10.9406104305243</v>
+        <v>10.27299393091428</v>
       </c>
     </row>
     <row r="149">
@@ -2267,10 +2267,10 @@
         <v>4</v>
       </c>
       <c r="C149" t="n">
-        <v>50.78798165267477</v>
+        <v>48.75143616441981</v>
       </c>
       <c r="D149" t="n">
-        <v>72.9168521097836</v>
+        <v>68.46732949153032</v>
       </c>
     </row>
     <row r="150">
@@ -2279,10 +2279,10 @@
         <v>5</v>
       </c>
       <c r="C150" t="n">
-        <v>75.21488842804288</v>
+        <v>72.19884926497319</v>
       </c>
       <c r="D150" t="n">
-        <v>53.69704773590538</v>
+        <v>50.42035350787413</v>
       </c>
     </row>
     <row r="151">
@@ -2291,10 +2291,10 @@
         <v>6</v>
       </c>
       <c r="C151" t="n">
-        <v>23.86171356220115</v>
+        <v>22.90488355014309</v>
       </c>
       <c r="D151" t="n">
-        <v>18.47485266998814</v>
+        <v>17.34748262526593</v>
       </c>
     </row>
     <row r="152">
@@ -2303,10 +2303,10 @@
         <v>7</v>
       </c>
       <c r="C152" t="n">
-        <v>50.70368594162364</v>
+        <v>48.6705206241184</v>
       </c>
       <c r="D152" t="n">
-        <v>216.1566852192408</v>
+        <v>202.966400228309</v>
       </c>
     </row>
     <row r="153">
@@ -2315,10 +2315,10 @@
         <v>8</v>
       </c>
       <c r="C153" t="n">
-        <v>46.14215021770806</v>
+        <v>44.29189776060323</v>
       </c>
       <c r="D153" t="n">
-        <v>57.62902033114246</v>
+        <v>54.11238978536508</v>
       </c>
     </row>
     <row r="154">
@@ -2327,10 +2327,10 @@
         <v>9</v>
       </c>
       <c r="C154" t="n">
-        <v>47.56389486199799</v>
+        <v>45.65663191645556</v>
       </c>
       <c r="D154" t="n">
-        <v>38.01277763477188</v>
+        <v>35.69316688671196</v>
       </c>
     </row>
     <row r="155">
@@ -2339,10 +2339,10 @@
         <v>10</v>
       </c>
       <c r="C155" t="n">
-        <v>72.79847540498726</v>
+        <v>69.87933190265714</v>
       </c>
       <c r="D155" t="n">
-        <v>42.42606811739712</v>
+        <v>39.83715013438145</v>
       </c>
     </row>
     <row r="156">
@@ -2351,10 +2351,10 @@
         <v>11</v>
       </c>
       <c r="C156" t="n">
-        <v>31.13003165795622</v>
+        <v>29.88174961446402</v>
       </c>
       <c r="D156" t="n">
-        <v>18.16354363922914</v>
+        <v>17.05517025348973</v>
       </c>
     </row>
     <row r="157">
@@ -2363,10 +2363,10 @@
         <v>12</v>
       </c>
       <c r="C157" t="n">
-        <v>67.04846671591856</v>
+        <v>64.35989260957727</v>
       </c>
       <c r="D157" t="n">
-        <v>25.74799133392534</v>
+        <v>24.17680077234708</v>
       </c>
     </row>
     <row r="158">
@@ -2377,10 +2377,10 @@
         <v>1</v>
       </c>
       <c r="C158" t="n">
-        <v>130.054111396106</v>
+        <v>124.8390761619031</v>
       </c>
       <c r="D158" t="n">
-        <v>230.8559867167859</v>
+        <v>216.7687228712627</v>
       </c>
     </row>
     <row r="159">
@@ -2389,10 +2389,10 @@
         <v>2</v>
       </c>
       <c r="C159" t="n">
-        <v>223.7671039496106</v>
+        <v>214.7942747262532</v>
       </c>
       <c r="D159" t="n">
-        <v>311.0132747994817</v>
+        <v>292.0346633981862</v>
       </c>
     </row>
     <row r="160">
@@ -2401,10 +2401,10 @@
         <v>3</v>
       </c>
       <c r="C160" t="n">
-        <v>182.4518648266455</v>
+        <v>175.1357339223405</v>
       </c>
       <c r="D160" t="n">
-        <v>319.4371100733703</v>
+        <v>299.9444604970975</v>
       </c>
     </row>
     <row r="161">
@@ -2413,10 +2413,10 @@
         <v>4</v>
       </c>
       <c r="C161" t="n">
-        <v>279.4072492769962</v>
+        <v>268.2033078250163</v>
       </c>
       <c r="D161" t="n">
-        <v>452.6846546527826</v>
+        <v>425.0609908283885</v>
       </c>
     </row>
     <row r="162">
@@ -2425,10 +2425,10 @@
         <v>5</v>
       </c>
       <c r="C162" t="n">
-        <v>168.3908888337431</v>
+        <v>161.6385885107484</v>
       </c>
       <c r="D162" t="n">
-        <v>296.1860670956371</v>
+        <v>278.1122396247349</v>
       </c>
     </row>
     <row r="163">
@@ -2437,10 +2437,10 @@
         <v>6</v>
       </c>
       <c r="C163" t="n">
-        <v>88.73166381978388</v>
+        <v>85.17361595615074</v>
       </c>
       <c r="D163" t="n">
-        <v>74.45671535048422</v>
+        <v>69.91322739883726</v>
       </c>
     </row>
     <row r="164">
@@ -2449,10 +2449,10 @@
         <v>7</v>
       </c>
       <c r="C164" t="n">
-        <v>27.03704045500077</v>
+        <v>25.95288312165852</v>
       </c>
       <c r="D164" t="n">
-        <v>18.47485266998814</v>
+        <v>17.34748262526593</v>
       </c>
     </row>
     <row r="165">
@@ -2461,10 +2461,10 @@
         <v>8</v>
       </c>
       <c r="C165" t="n">
-        <v>72.18604300256146</v>
+        <v>69.29145740557499</v>
       </c>
       <c r="D165" t="n">
-        <v>32.62924451679817</v>
+        <v>30.63814702296477</v>
       </c>
     </row>
     <row r="166">
@@ -2473,10 +2473,10 @@
         <v>9</v>
       </c>
       <c r="C166" t="n">
-        <v>54.69657446366934</v>
+        <v>52.50329844989176</v>
       </c>
       <c r="D166" t="n">
-        <v>8.087278941941969</v>
+        <v>7.593778063460326</v>
       </c>
     </row>
     <row r="167">
@@ -2485,10 +2485,10 @@
         <v>10</v>
       </c>
       <c r="C167" t="n">
-        <v>95.76412734111437</v>
+        <v>91.92408497032349</v>
       </c>
       <c r="D167" t="n">
-        <v>108.7351215874265</v>
+        <v>102.0999012110266</v>
       </c>
     </row>
     <row r="168">
@@ -2497,10 +2497,10 @@
         <v>11</v>
       </c>
       <c r="C168" t="n">
-        <v>238.1094363975246</v>
+        <v>228.5614944902728</v>
       </c>
       <c r="D168" t="n">
-        <v>234.3416436900954</v>
+        <v>220.041678540368</v>
       </c>
     </row>
     <row r="169">
@@ -2509,10 +2509,10 @@
         <v>12</v>
       </c>
       <c r="C169" t="n">
-        <v>366.8109803589832</v>
+        <v>352.102239771472</v>
       </c>
       <c r="D169" t="n">
-        <v>138.6683240608168</v>
+        <v>130.2065237157482</v>
       </c>
     </row>
     <row r="170">
@@ -2523,10 +2523,10 @@
         <v>1</v>
       </c>
       <c r="C170" t="n">
-        <v>138.5250234574885</v>
+        <v>132.9703134187622</v>
       </c>
       <c r="D170" t="n">
-        <v>155.5890175506625</v>
+        <v>146.0946848592134</v>
       </c>
     </row>
     <row r="171">
@@ -2535,10 +2535,10 @@
         <v>2</v>
       </c>
       <c r="C171" t="n">
-        <v>19.18354178476588</v>
+        <v>18.41430161811204</v>
       </c>
       <c r="D171" t="n">
-        <v>39.6483261777854</v>
+        <v>37.22891120032136</v>
       </c>
     </row>
     <row r="172">
@@ -2547,10 +2547,10 @@
         <v>3</v>
       </c>
       <c r="C172" t="n">
-        <v>138.3690050115393</v>
+        <v>132.8205511509843</v>
       </c>
       <c r="D172" t="n">
-        <v>337.7907722063459</v>
+        <v>317.1781478584592</v>
       </c>
     </row>
     <row r="173">
@@ -2559,10 +2559,10 @@
         <v>4</v>
       </c>
       <c r="C173" t="n">
-        <v>146.5056351425879</v>
+        <v>140.6309108368652</v>
       </c>
       <c r="D173" t="n">
-        <v>68.54384652597561</v>
+        <v>64.36117288284822</v>
       </c>
     </row>
     <row r="174">
@@ -2571,10 +2571,10 @@
         <v>5</v>
       </c>
       <c r="C174" t="n">
-        <v>238.5826328562362</v>
+        <v>229.0157162608457</v>
       </c>
       <c r="D174" t="n">
-        <v>115.9492205737614</v>
+        <v>108.8737823919948</v>
       </c>
     </row>
     <row r="175">
@@ -2583,10 +2583,10 @@
         <v>6</v>
       </c>
       <c r="C175" t="n">
-        <v>127.4696539008041</v>
+        <v>122.3582527367172</v>
       </c>
       <c r="D175" t="n">
-        <v>85.3644174278279</v>
+        <v>80.15532110579714</v>
       </c>
     </row>
     <row r="176">
@@ -2595,10 +2595,10 @@
         <v>7</v>
       </c>
       <c r="C176" t="n">
-        <v>266.311292779793</v>
+        <v>255.6324856263396</v>
       </c>
       <c r="D176" t="n">
-        <v>229.3232959644335</v>
+        <v>215.3295597736575</v>
       </c>
     </row>
     <row r="177">
@@ -2607,10 +2607,10 @@
         <v>8</v>
       </c>
       <c r="C177" t="n">
-        <v>214.3660754492314</v>
+        <v>205.7702177367392</v>
       </c>
       <c r="D177" t="n">
-        <v>332.3302607126742</v>
+        <v>312.0508469833938</v>
       </c>
     </row>
     <row r="178">
@@ -2619,10 +2619,10 @@
         <v>9</v>
       </c>
       <c r="C178" t="n">
-        <v>41.61050863877016</v>
+        <v>39.94197031779873</v>
       </c>
       <c r="D178" t="n">
-        <v>32.65636873921438</v>
+        <v>30.6636160746262</v>
       </c>
     </row>
     <row r="179">
@@ -2631,10 +2631,10 @@
         <v>10</v>
       </c>
       <c r="C179" t="n">
-        <v>86.56085900738998</v>
+        <v>83.08985816950394</v>
       </c>
       <c r="D179" t="n">
-        <v>35.39931165340919</v>
+        <v>33.23917948484966</v>
       </c>
     </row>
     <row r="180">
@@ -2643,10 +2643,10 @@
         <v>11</v>
       </c>
       <c r="C180" t="n">
-        <v>154.5419536232181</v>
+        <v>148.3449812656662</v>
       </c>
       <c r="D180" t="n">
-        <v>110.401857185292</v>
+        <v>103.6649294871034</v>
       </c>
     </row>
     <row r="181">
@@ -2655,10 +2655,10 @@
         <v>12</v>
       </c>
       <c r="C181" t="n">
-        <v>81.39143276740769</v>
+        <v>78.1277205703245</v>
       </c>
       <c r="D181" t="n">
-        <v>56.21390544740409</v>
+        <v>52.78362785708811</v>
       </c>
     </row>
     <row r="182">
@@ -2669,10 +2669,10 @@
         <v>1</v>
       </c>
       <c r="C182" t="n">
-        <v>282.8091922157575</v>
+        <v>271.4688363736446</v>
       </c>
       <c r="D182" t="n">
-        <v>234.382968184846</v>
+        <v>220.0804813372017</v>
       </c>
     </row>
     <row r="183">
@@ -2681,10 +2681,10 @@
         <v>2</v>
       </c>
       <c r="C183" t="n">
-        <v>223.694548747105</v>
+        <v>214.7246289122585</v>
       </c>
       <c r="D183" t="n">
-        <v>87.16670922016313</v>
+        <v>81.84763368396366</v>
       </c>
     </row>
     <row r="184">
@@ -2693,10 +2693,10 @@
         <v>3</v>
       </c>
       <c r="C184" t="n">
-        <v>221.82924329302</v>
+        <v>212.9341202759071</v>
       </c>
       <c r="D184" t="n">
-        <v>228.4716575834568</v>
+        <v>214.5298899586444</v>
       </c>
     </row>
     <row r="185">
@@ -2705,10 +2705,10 @@
         <v>4</v>
       </c>
       <c r="C185" t="n">
-        <v>208.2656198553328</v>
+        <v>199.9143840969284</v>
       </c>
       <c r="D185" t="n">
-        <v>424.8897552541068</v>
+        <v>398.9621881476603</v>
       </c>
     </row>
     <row r="186">
@@ -2717,10 +2717,10 @@
         <v>5</v>
       </c>
       <c r="C186" t="n">
-        <v>97.28438650698861</v>
+        <v>93.3833833174274</v>
       </c>
       <c r="D186" t="n">
-        <v>94.18341050773667</v>
+        <v>88.4361627427419</v>
       </c>
     </row>
     <row r="187">
@@ -2729,10 +2729,10 @@
         <v>6</v>
       </c>
       <c r="C187" t="n">
-        <v>142.5020815823688</v>
+        <v>136.7878956299087</v>
       </c>
       <c r="D187" t="n">
-        <v>77.94062601913652</v>
+        <v>73.18454332605992</v>
       </c>
     </row>
     <row r="188">
@@ -2741,10 +2741,10 @@
         <v>7</v>
       </c>
       <c r="C188" t="n">
-        <v>249.665978335058</v>
+        <v>239.6546310595112</v>
       </c>
       <c r="D188" t="n">
-        <v>154.5870773209822</v>
+        <v>145.1538848952619</v>
       </c>
     </row>
     <row r="189">
@@ -2753,10 +2753,10 @@
         <v>8</v>
       </c>
       <c r="C189" t="n">
-        <v>91.56636215191168</v>
+        <v>87.89464581965662</v>
       </c>
       <c r="D189" t="n">
-        <v>71.01181003024752</v>
+        <v>66.67853664075767</v>
       </c>
     </row>
     <row r="190">
@@ -2765,10 +2765,10 @@
         <v>9</v>
       </c>
       <c r="C190" t="n">
-        <v>178.9106802438269</v>
+        <v>171.7365471754378</v>
       </c>
       <c r="D190" t="n">
-        <v>73.29801033776202</v>
+        <v>68.82522873194343</v>
       </c>
     </row>
     <row r="191">
@@ -2777,10 +2777,10 @@
         <v>10</v>
       </c>
       <c r="C191" t="n">
-        <v>269.3587834658959</v>
+        <v>258.5577750907102</v>
       </c>
       <c r="D191" t="n">
-        <v>200.7827665721997</v>
+        <v>188.5306268353747</v>
       </c>
     </row>
     <row r="192">
@@ -2789,10 +2789,10 @@
         <v>11</v>
       </c>
       <c r="C192" t="n">
-        <v>59.68659206882781</v>
+        <v>57.29322151477893</v>
       </c>
       <c r="D192" t="n">
-        <v>40.98561765733415</v>
+        <v>38.48459865400665</v>
       </c>
     </row>
     <row r="193">
@@ -2801,10 +2801,10 @@
         <v>12</v>
       </c>
       <c r="C193" t="n">
-        <v>312.1049443212432</v>
+        <v>299.5898591468351</v>
       </c>
       <c r="D193" t="n">
-        <v>206.2378981065315</v>
+        <v>193.6528760462758</v>
       </c>
     </row>
     <row r="194">
@@ -2815,10 +2815,10 @@
         <v>1</v>
       </c>
       <c r="C194" t="n">
-        <v>133.4916659724814</v>
+        <v>128.1387883583426</v>
       </c>
       <c r="D194" t="n">
-        <v>87.69314709957401</v>
+        <v>82.34194733990948</v>
       </c>
     </row>
     <row r="195">
@@ -2827,10 +2827,10 @@
         <v>2</v>
       </c>
       <c r="C195" t="n">
-        <v>5.068305067021176</v>
+        <v>4.865071280572837</v>
       </c>
       <c r="D195" t="n">
-        <v>6.826494886212494</v>
+        <v>6.409929407578546</v>
       </c>
     </row>
     <row r="196">
@@ -2839,10 +2839,10 @@
         <v>3</v>
       </c>
       <c r="C196" t="n">
-        <v>36.92426037917923</v>
+        <v>35.44363576218563</v>
       </c>
       <c r="D196" t="n">
-        <v>34.42623550101468</v>
+        <v>32.32548225823274</v>
       </c>
     </row>
     <row r="197">
@@ -2851,10 +2851,10 @@
         <v>4</v>
       </c>
       <c r="C197" t="n">
-        <v>53.40536506929195</v>
+        <v>51.26386521556134</v>
       </c>
       <c r="D197" t="n">
-        <v>46.47245510415657</v>
+        <v>43.63661902335078</v>
       </c>
     </row>
     <row r="198">
@@ -2863,10 +2863,10 @@
         <v>5</v>
       </c>
       <c r="C198" t="n">
-        <v>85.12648741219544</v>
+        <v>81.71300339040678</v>
       </c>
       <c r="D198" t="n">
-        <v>85.07160547984125</v>
+        <v>79.88037709022616</v>
       </c>
     </row>
     <row r="199">
@@ -2875,10 +2875,10 @@
         <v>6</v>
       </c>
       <c r="C199" t="n">
-        <v>8.648775522544419</v>
+        <v>8.301968577353671</v>
       </c>
       <c r="D199" t="n">
-        <v>4.958547076191262</v>
+        <v>4.655967264655125</v>
       </c>
     </row>
     <row r="200">
@@ -2887,10 +2887,10 @@
         <v>7</v>
       </c>
       <c r="C200" t="n">
-        <v>37.70757563485872</v>
+        <v>36.19554088700494</v>
       </c>
       <c r="D200" t="n">
-        <v>89.83734074233129</v>
+        <v>84.35529827847272</v>
       </c>
     </row>
     <row r="201">
@@ -2899,10 +2899,10 @@
         <v>8</v>
       </c>
       <c r="C201" t="n">
-        <v>109.0902444047529</v>
+        <v>104.7158385349849</v>
       </c>
       <c r="D201" t="n">
-        <v>40.05258783352926</v>
+        <v>37.60850405415074</v>
       </c>
     </row>
     <row r="202">
@@ -2911,10 +2911,10 @@
         <v>9</v>
       </c>
       <c r="C202" t="n">
-        <v>91.84108447473984</v>
+        <v>88.15835206173352</v>
       </c>
       <c r="D202" t="n">
-        <v>59.83791870167174</v>
+        <v>56.18649704825994</v>
       </c>
     </row>
     <row r="203">
@@ -2923,10 +2923,10 @@
         <v>10</v>
       </c>
       <c r="C203" t="n">
-        <v>27.72924911001008</v>
+        <v>26.61733492618043</v>
       </c>
       <c r="D203" t="n">
-        <v>48.72098879828846</v>
+        <v>45.74794298831222</v>
       </c>
     </row>
     <row r="204">
@@ -2935,10 +2935,10 @@
         <v>11</v>
       </c>
       <c r="C204" t="n">
-        <v>36.86782180056895</v>
+        <v>35.38946031215208</v>
       </c>
       <c r="D204" t="n">
-        <v>57.90301665041671</v>
+        <v>54.3696663370595</v>
       </c>
     </row>
     <row r="205">
@@ -2947,10 +2947,10 @@
         <v>12</v>
       </c>
       <c r="C205" t="n">
-        <v>60.10621859736482</v>
+        <v>57.69602145392147</v>
       </c>
       <c r="D205" t="n">
-        <v>46.90798584878765</v>
+        <v>44.04557286781256</v>
       </c>
     </row>
     <row r="206">
@@ -2961,10 +2961,10 @@
         <v>1</v>
       </c>
       <c r="C206" t="n">
-        <v>303.309916546203</v>
+        <v>309.7835191284429</v>
       </c>
       <c r="D206" t="n">
-        <v>314.7676310233977</v>
+        <v>322.635987468936</v>
       </c>
     </row>
     <row r="207">
@@ -2973,10 +2973,10 @@
         <v>2</v>
       </c>
       <c r="C207" t="n">
-        <v>210.5653181342403</v>
+        <v>210.9097741101004</v>
       </c>
       <c r="D207" t="n">
-        <v>195.278272580785</v>
+        <v>191.3342894157855</v>
       </c>
     </row>
     <row r="208">
@@ -2985,10 +2985,10 @@
         <v>3</v>
       </c>
       <c r="C208" t="n">
-        <v>223.9022592502805</v>
+        <v>229.7468646846923</v>
       </c>
       <c r="D208" t="n">
-        <v>238.0282084559564</v>
+        <v>247.4464505426254</v>
       </c>
     </row>
     <row r="209">
@@ -2997,10 +2997,10 @@
         <v>4</v>
       </c>
       <c r="C209" t="n">
-        <v>539.9628587258261</v>
+        <v>579.8225042682515</v>
       </c>
       <c r="D209" t="n">
-        <v>665.4885268439618</v>
+        <v>744.5144555872507</v>
       </c>
     </row>
     <row r="210">
@@ -3009,10 +3009,10 @@
         <v>5</v>
       </c>
       <c r="C210" t="n">
-        <v>301.3220593222113</v>
+        <v>323.9040722399145</v>
       </c>
       <c r="D210" t="n">
-        <v>293.4372096909116</v>
+        <v>344.4132738630638</v>
       </c>
     </row>
     <row r="211">
@@ -3021,10 +3021,10 @@
         <v>6</v>
       </c>
       <c r="C211" t="n">
-        <v>1058.702037133946</v>
+        <v>1092.381511462321</v>
       </c>
       <c r="D211" t="n">
-        <v>1080.911394641637</v>
+        <v>1130.208687122463</v>
       </c>
     </row>
     <row r="212">
@@ -3033,10 +3033,10 @@
         <v>7</v>
       </c>
       <c r="C212" t="n">
-        <v>519.5050613688212</v>
+        <v>577.9061840186755</v>
       </c>
       <c r="D212" t="n">
-        <v>605.93607903236</v>
+        <v>728.8416755722365</v>
       </c>
     </row>
     <row r="213">
@@ -3045,10 +3045,10 @@
         <v>8</v>
       </c>
       <c r="C213" t="n">
-        <v>580.0360790225873</v>
+        <v>606.4417544570731</v>
       </c>
       <c r="D213" t="n">
-        <v>615.4985920135333</v>
+        <v>659.9700683829057</v>
       </c>
     </row>
     <row r="214">
@@ -3057,10 +3057,10 @@
         <v>9</v>
       </c>
       <c r="C214" t="n">
-        <v>273.4741789217958</v>
+        <v>285.7115639057716</v>
       </c>
       <c r="D214" t="n">
-        <v>295.2330055624921</v>
+        <v>317.7215319255458</v>
       </c>
     </row>
     <row r="215">
@@ -3069,10 +3069,10 @@
         <v>10</v>
       </c>
       <c r="C215" t="n">
-        <v>1236.489531813095</v>
+        <v>1283.991238409127</v>
       </c>
       <c r="D215" t="n">
-        <v>1274.319428616542</v>
+        <v>1358.831004966153</v>
       </c>
     </row>
     <row r="216">
@@ -3081,10 +3081,10 @@
         <v>11</v>
       </c>
       <c r="C216" t="n">
-        <v>679.8080610834414</v>
+        <v>735.1983154370909</v>
       </c>
       <c r="D216" t="n">
-        <v>642.6605360744878</v>
+        <v>690.1398384821941</v>
       </c>
     </row>
     <row r="217">
@@ -3093,10 +3093,10 @@
         <v>12</v>
       </c>
       <c r="C217" t="n">
-        <v>510.8143752041662</v>
+        <v>524.809689462469</v>
       </c>
       <c r="D217" t="n">
-        <v>370.204056969939</v>
+        <v>391.1784130123241</v>
       </c>
     </row>
     <row r="218">
@@ -3107,10 +3107,10 @@
         <v>1</v>
       </c>
       <c r="C218" t="n">
-        <v>464.8950456627734</v>
+        <v>473.7725607297504</v>
       </c>
       <c r="D218" t="n">
-        <v>404.8897658632732</v>
+        <v>414.4943581737198</v>
       </c>
     </row>
     <row r="219">
@@ -3119,10 +3119,10 @@
         <v>2</v>
       </c>
       <c r="C219" t="n">
-        <v>627.4926359854262</v>
+        <v>640.3798007991006</v>
       </c>
       <c r="D219" t="n">
-        <v>489.8935866563978</v>
+        <v>504.8941966297115</v>
       </c>
     </row>
     <row r="220">
@@ -3131,10 +3131,10 @@
         <v>3</v>
       </c>
       <c r="C220" t="n">
-        <v>985.5116154818029</v>
+        <v>1000.378889002457</v>
       </c>
       <c r="D220" t="n">
-        <v>700.8527040648374</v>
+        <v>715.1490376091863</v>
       </c>
     </row>
     <row r="221">
@@ -3143,10 +3143,10 @@
         <v>4</v>
       </c>
       <c r="C221" t="n">
-        <v>280.2039064675896</v>
+        <v>285.6585576268807</v>
       </c>
       <c r="D221" t="n">
-        <v>327.8542962271332</v>
+        <v>331.901936212599</v>
       </c>
     </row>
     <row r="222">
@@ -3155,10 +3155,10 @@
         <v>5</v>
       </c>
       <c r="C222" t="n">
-        <v>681.375769447817</v>
+        <v>713.4781430431922</v>
       </c>
       <c r="D222" t="n">
-        <v>570.4725314266174</v>
+        <v>630.0790214268379</v>
       </c>
     </row>
     <row r="223">
@@ -3167,10 +3167,10 @@
         <v>6</v>
       </c>
       <c r="C223" t="n">
-        <v>403.9691894022718</v>
+        <v>409.502496864833</v>
       </c>
       <c r="D223" t="n">
-        <v>317.9251592921427</v>
+        <v>322.6372147862144</v>
       </c>
     </row>
     <row r="224">
@@ -3179,10 +3179,10 @@
         <v>7</v>
       </c>
       <c r="C224" t="n">
-        <v>341.1166065130264</v>
+        <v>368.2606017061975</v>
       </c>
       <c r="D224" t="n">
-        <v>399.5376876214065</v>
+        <v>450.8448921081423</v>
       </c>
     </row>
     <row r="225">
@@ -3191,10 +3191,10 @@
         <v>8</v>
       </c>
       <c r="C225" t="n">
-        <v>416.4458724439396</v>
+        <v>436.1882173467339</v>
       </c>
       <c r="D225" t="n">
-        <v>290.2774520416102</v>
+        <v>325.236181179027</v>
       </c>
     </row>
     <row r="226">
@@ -3203,10 +3203,10 @@
         <v>9</v>
       </c>
       <c r="C226" t="n">
-        <v>469.8234273737044</v>
+        <v>477.2778494951258</v>
       </c>
       <c r="D226" t="n">
-        <v>323.8043958357738</v>
+        <v>332.1087449927961</v>
       </c>
     </row>
   </sheetData>

</xml_diff>